<commit_message>
feat(excel): Von/Bis nur Datum, Uhrzeiten ausschliesslich im Zeiten-Blatt
Das Termine-Blatt ist tagesgenau. Wer eine Uhrzeit braucht, traegt im Blatt
'Zeiten' einen Block ein - damit gibt es genau einen Ort fuer Uhrzeiten.

- Vorlage: Von/Bis als Datum, Zahlenformat DD.MM.YYYY
- Parser: eine Datumszelle kommt als datetime 00:00 zurueck; ohne
  Unterscheidung waere 'Bis' ebenfalls Mitternacht und der Termin null
  Stunden lang. Jetzt wird daraus 23:59.
- Konverter: schreibt nur Datum und verschiebt Uhrzeiten aus alten Dateien
  ins Blatt 'Zeiten'; unbekannte Pruefstaende kommen in die Stammliste.
- Anleitung nennt die neue Regel.
</commit_message>
<xml_diff>
--- a/terminboard/vorlagen/termine_modell2.xlsx
+++ b/terminboard/vorlagen/termine_modell2.xlsx
@@ -22,9 +22,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="DD.MM.YYYY HH:MM"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="DD.MM.YYYY HH:MM"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -69,12 +71,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -507,10 +510,10 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>46328.29166666666</v>
+        <v>46328</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>46328.625</v>
+        <v>46328</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -538,10 +541,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>46342.33333333334</v>
+        <v>46342</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46347.66666666666</v>
+        <v>46347</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -569,10 +572,10 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>46344.25</v>
+        <v>46344</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>46345.75</v>
+        <v>46345</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -600,10 +603,10 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>46350.375</v>
+        <v>46350</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>46350.54166666666</v>
+        <v>46350</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -631,10 +634,10 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>46353.41666666666</v>
+        <v>46353</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>46353.5</v>
+        <v>46353</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -662,7 +665,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>46357.33333333334</v>
+        <v>46357</v>
       </c>
       <c r="E7" s="2" t="n"/>
       <c r="F7" t="inlineStr">
@@ -2703,17 +2706,17 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>46342.33333333334</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>46342.5</v>
+        <v>4</v>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>46350.375</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>46350.54166666666</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tag 1, vormittags</t>
+          <t>Halbtag, Rest des Tages freigegeben</t>
         </is>
       </c>
     </row>
@@ -2721,15 +2724,15 @@
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>46343.33333333334</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>46343.66666666666</v>
+      <c r="B3" s="3" t="n">
+        <v>46342.33333333334</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>46342.5</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Tag 2, ganztags</t>
+          <t>Tag 1, vormittags</t>
         </is>
       </c>
     </row>
@@ -2737,15 +2740,15 @@
       <c r="A4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>46345.29166666666</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>46345.45833333334</v>
+      <c r="B4" s="3" t="n">
+        <v>46343.33333333334</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>46343.66666666666</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Tag 4, vormittags</t>
+          <t>Tag 2, ganztags</t>
         </is>
       </c>
     </row>
@@ -2753,1997 +2756,2009 @@
       <c r="A5" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
+        <v>46345.29166666666</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>46345.45833333334</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Tag 4, vormittags</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="n">
         <v>46346.33333333334</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C6" s="3" t="n">
         <v>46346.58333333334</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Tag 5, 6 Stunden</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-    </row>
     <row r="7">
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
+      <c r="B14" s="3" t="n"/>
+      <c r="C14" s="3" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="2" t="n"/>
+      <c r="B18" s="3" t="n"/>
+      <c r="C18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
+      <c r="B20" s="3" t="n"/>
+      <c r="C20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="2" t="n"/>
-      <c r="C21" s="2" t="n"/>
+      <c r="B21" s="3" t="n"/>
+      <c r="C21" s="3" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
+      <c r="B22" s="3" t="n"/>
+      <c r="C22" s="3" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="2" t="n"/>
-      <c r="C23" s="2" t="n"/>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="2" t="n"/>
+      <c r="B24" s="3" t="n"/>
+      <c r="C24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="n"/>
+      <c r="B27" s="3" t="n"/>
+      <c r="C27" s="3" t="n"/>
     </row>
     <row r="28">
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
+      <c r="B28" s="3" t="n"/>
+      <c r="C28" s="3" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
+      <c r="B29" s="3" t="n"/>
+      <c r="C29" s="3" t="n"/>
     </row>
     <row r="30">
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
+      <c r="B30" s="3" t="n"/>
+      <c r="C30" s="3" t="n"/>
     </row>
     <row r="31">
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
+      <c r="B31" s="3" t="n"/>
+      <c r="C31" s="3" t="n"/>
     </row>
     <row r="32">
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
+      <c r="B32" s="3" t="n"/>
+      <c r="C32" s="3" t="n"/>
     </row>
     <row r="33">
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
+      <c r="B33" s="3" t="n"/>
+      <c r="C33" s="3" t="n"/>
     </row>
     <row r="34">
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="n"/>
+      <c r="B34" s="3" t="n"/>
+      <c r="C34" s="3" t="n"/>
     </row>
     <row r="35">
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
+      <c r="B35" s="3" t="n"/>
+      <c r="C35" s="3" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
+      <c r="B36" s="3" t="n"/>
+      <c r="C36" s="3" t="n"/>
     </row>
     <row r="37">
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="2" t="n"/>
+      <c r="B37" s="3" t="n"/>
+      <c r="C37" s="3" t="n"/>
     </row>
     <row r="38">
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
+      <c r="B38" s="3" t="n"/>
+      <c r="C38" s="3" t="n"/>
     </row>
     <row r="39">
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="2" t="n"/>
+      <c r="B39" s="3" t="n"/>
+      <c r="C39" s="3" t="n"/>
     </row>
     <row r="40">
-      <c r="B40" s="2" t="n"/>
-      <c r="C40" s="2" t="n"/>
+      <c r="B40" s="3" t="n"/>
+      <c r="C40" s="3" t="n"/>
     </row>
     <row r="41">
-      <c r="B41" s="2" t="n"/>
-      <c r="C41" s="2" t="n"/>
+      <c r="B41" s="3" t="n"/>
+      <c r="C41" s="3" t="n"/>
     </row>
     <row r="42">
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="2" t="n"/>
+      <c r="B42" s="3" t="n"/>
+      <c r="C42" s="3" t="n"/>
     </row>
     <row r="43">
-      <c r="B43" s="2" t="n"/>
-      <c r="C43" s="2" t="n"/>
+      <c r="B43" s="3" t="n"/>
+      <c r="C43" s="3" t="n"/>
     </row>
     <row r="44">
-      <c r="B44" s="2" t="n"/>
-      <c r="C44" s="2" t="n"/>
+      <c r="B44" s="3" t="n"/>
+      <c r="C44" s="3" t="n"/>
     </row>
     <row r="45">
-      <c r="B45" s="2" t="n"/>
-      <c r="C45" s="2" t="n"/>
+      <c r="B45" s="3" t="n"/>
+      <c r="C45" s="3" t="n"/>
     </row>
     <row r="46">
-      <c r="B46" s="2" t="n"/>
-      <c r="C46" s="2" t="n"/>
+      <c r="B46" s="3" t="n"/>
+      <c r="C46" s="3" t="n"/>
     </row>
     <row r="47">
-      <c r="B47" s="2" t="n"/>
-      <c r="C47" s="2" t="n"/>
+      <c r="B47" s="3" t="n"/>
+      <c r="C47" s="3" t="n"/>
     </row>
     <row r="48">
-      <c r="B48" s="2" t="n"/>
-      <c r="C48" s="2" t="n"/>
+      <c r="B48" s="3" t="n"/>
+      <c r="C48" s="3" t="n"/>
     </row>
     <row r="49">
-      <c r="B49" s="2" t="n"/>
-      <c r="C49" s="2" t="n"/>
+      <c r="B49" s="3" t="n"/>
+      <c r="C49" s="3" t="n"/>
     </row>
     <row r="50">
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="2" t="n"/>
+      <c r="B50" s="3" t="n"/>
+      <c r="C50" s="3" t="n"/>
     </row>
     <row r="51">
-      <c r="B51" s="2" t="n"/>
-      <c r="C51" s="2" t="n"/>
+      <c r="B51" s="3" t="n"/>
+      <c r="C51" s="3" t="n"/>
     </row>
     <row r="52">
-      <c r="B52" s="2" t="n"/>
-      <c r="C52" s="2" t="n"/>
+      <c r="B52" s="3" t="n"/>
+      <c r="C52" s="3" t="n"/>
     </row>
     <row r="53">
-      <c r="B53" s="2" t="n"/>
-      <c r="C53" s="2" t="n"/>
+      <c r="B53" s="3" t="n"/>
+      <c r="C53" s="3" t="n"/>
     </row>
     <row r="54">
-      <c r="B54" s="2" t="n"/>
-      <c r="C54" s="2" t="n"/>
+      <c r="B54" s="3" t="n"/>
+      <c r="C54" s="3" t="n"/>
     </row>
     <row r="55">
-      <c r="B55" s="2" t="n"/>
-      <c r="C55" s="2" t="n"/>
+      <c r="B55" s="3" t="n"/>
+      <c r="C55" s="3" t="n"/>
     </row>
     <row r="56">
-      <c r="B56" s="2" t="n"/>
-      <c r="C56" s="2" t="n"/>
+      <c r="B56" s="3" t="n"/>
+      <c r="C56" s="3" t="n"/>
     </row>
     <row r="57">
-      <c r="B57" s="2" t="n"/>
-      <c r="C57" s="2" t="n"/>
+      <c r="B57" s="3" t="n"/>
+      <c r="C57" s="3" t="n"/>
     </row>
     <row r="58">
-      <c r="B58" s="2" t="n"/>
-      <c r="C58" s="2" t="n"/>
+      <c r="B58" s="3" t="n"/>
+      <c r="C58" s="3" t="n"/>
     </row>
     <row r="59">
-      <c r="B59" s="2" t="n"/>
-      <c r="C59" s="2" t="n"/>
+      <c r="B59" s="3" t="n"/>
+      <c r="C59" s="3" t="n"/>
     </row>
     <row r="60">
-      <c r="B60" s="2" t="n"/>
-      <c r="C60" s="2" t="n"/>
+      <c r="B60" s="3" t="n"/>
+      <c r="C60" s="3" t="n"/>
     </row>
     <row r="61">
-      <c r="B61" s="2" t="n"/>
-      <c r="C61" s="2" t="n"/>
+      <c r="B61" s="3" t="n"/>
+      <c r="C61" s="3" t="n"/>
     </row>
     <row r="62">
-      <c r="B62" s="2" t="n"/>
-      <c r="C62" s="2" t="n"/>
+      <c r="B62" s="3" t="n"/>
+      <c r="C62" s="3" t="n"/>
     </row>
     <row r="63">
-      <c r="B63" s="2" t="n"/>
-      <c r="C63" s="2" t="n"/>
+      <c r="B63" s="3" t="n"/>
+      <c r="C63" s="3" t="n"/>
     </row>
     <row r="64">
-      <c r="B64" s="2" t="n"/>
-      <c r="C64" s="2" t="n"/>
+      <c r="B64" s="3" t="n"/>
+      <c r="C64" s="3" t="n"/>
     </row>
     <row r="65">
-      <c r="B65" s="2" t="n"/>
-      <c r="C65" s="2" t="n"/>
+      <c r="B65" s="3" t="n"/>
+      <c r="C65" s="3" t="n"/>
     </row>
     <row r="66">
-      <c r="B66" s="2" t="n"/>
-      <c r="C66" s="2" t="n"/>
+      <c r="B66" s="3" t="n"/>
+      <c r="C66" s="3" t="n"/>
     </row>
     <row r="67">
-      <c r="B67" s="2" t="n"/>
-      <c r="C67" s="2" t="n"/>
+      <c r="B67" s="3" t="n"/>
+      <c r="C67" s="3" t="n"/>
     </row>
     <row r="68">
-      <c r="B68" s="2" t="n"/>
-      <c r="C68" s="2" t="n"/>
+      <c r="B68" s="3" t="n"/>
+      <c r="C68" s="3" t="n"/>
     </row>
     <row r="69">
-      <c r="B69" s="2" t="n"/>
-      <c r="C69" s="2" t="n"/>
+      <c r="B69" s="3" t="n"/>
+      <c r="C69" s="3" t="n"/>
     </row>
     <row r="70">
-      <c r="B70" s="2" t="n"/>
-      <c r="C70" s="2" t="n"/>
+      <c r="B70" s="3" t="n"/>
+      <c r="C70" s="3" t="n"/>
     </row>
     <row r="71">
-      <c r="B71" s="2" t="n"/>
-      <c r="C71" s="2" t="n"/>
+      <c r="B71" s="3" t="n"/>
+      <c r="C71" s="3" t="n"/>
     </row>
     <row r="72">
-      <c r="B72" s="2" t="n"/>
-      <c r="C72" s="2" t="n"/>
+      <c r="B72" s="3" t="n"/>
+      <c r="C72" s="3" t="n"/>
     </row>
     <row r="73">
-      <c r="B73" s="2" t="n"/>
-      <c r="C73" s="2" t="n"/>
+      <c r="B73" s="3" t="n"/>
+      <c r="C73" s="3" t="n"/>
     </row>
     <row r="74">
-      <c r="B74" s="2" t="n"/>
-      <c r="C74" s="2" t="n"/>
+      <c r="B74" s="3" t="n"/>
+      <c r="C74" s="3" t="n"/>
     </row>
     <row r="75">
-      <c r="B75" s="2" t="n"/>
-      <c r="C75" s="2" t="n"/>
+      <c r="B75" s="3" t="n"/>
+      <c r="C75" s="3" t="n"/>
     </row>
     <row r="76">
-      <c r="B76" s="2" t="n"/>
-      <c r="C76" s="2" t="n"/>
+      <c r="B76" s="3" t="n"/>
+      <c r="C76" s="3" t="n"/>
     </row>
     <row r="77">
-      <c r="B77" s="2" t="n"/>
-      <c r="C77" s="2" t="n"/>
+      <c r="B77" s="3" t="n"/>
+      <c r="C77" s="3" t="n"/>
     </row>
     <row r="78">
-      <c r="B78" s="2" t="n"/>
-      <c r="C78" s="2" t="n"/>
+      <c r="B78" s="3" t="n"/>
+      <c r="C78" s="3" t="n"/>
     </row>
     <row r="79">
-      <c r="B79" s="2" t="n"/>
-      <c r="C79" s="2" t="n"/>
+      <c r="B79" s="3" t="n"/>
+      <c r="C79" s="3" t="n"/>
     </row>
     <row r="80">
-      <c r="B80" s="2" t="n"/>
-      <c r="C80" s="2" t="n"/>
+      <c r="B80" s="3" t="n"/>
+      <c r="C80" s="3" t="n"/>
     </row>
     <row r="81">
-      <c r="B81" s="2" t="n"/>
-      <c r="C81" s="2" t="n"/>
+      <c r="B81" s="3" t="n"/>
+      <c r="C81" s="3" t="n"/>
     </row>
     <row r="82">
-      <c r="B82" s="2" t="n"/>
-      <c r="C82" s="2" t="n"/>
+      <c r="B82" s="3" t="n"/>
+      <c r="C82" s="3" t="n"/>
     </row>
     <row r="83">
-      <c r="B83" s="2" t="n"/>
-      <c r="C83" s="2" t="n"/>
+      <c r="B83" s="3" t="n"/>
+      <c r="C83" s="3" t="n"/>
     </row>
     <row r="84">
-      <c r="B84" s="2" t="n"/>
-      <c r="C84" s="2" t="n"/>
+      <c r="B84" s="3" t="n"/>
+      <c r="C84" s="3" t="n"/>
     </row>
     <row r="85">
-      <c r="B85" s="2" t="n"/>
-      <c r="C85" s="2" t="n"/>
+      <c r="B85" s="3" t="n"/>
+      <c r="C85" s="3" t="n"/>
     </row>
     <row r="86">
-      <c r="B86" s="2" t="n"/>
-      <c r="C86" s="2" t="n"/>
+      <c r="B86" s="3" t="n"/>
+      <c r="C86" s="3" t="n"/>
     </row>
     <row r="87">
-      <c r="B87" s="2" t="n"/>
-      <c r="C87" s="2" t="n"/>
+      <c r="B87" s="3" t="n"/>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
-      <c r="B88" s="2" t="n"/>
-      <c r="C88" s="2" t="n"/>
+      <c r="B88" s="3" t="n"/>
+      <c r="C88" s="3" t="n"/>
     </row>
     <row r="89">
-      <c r="B89" s="2" t="n"/>
-      <c r="C89" s="2" t="n"/>
+      <c r="B89" s="3" t="n"/>
+      <c r="C89" s="3" t="n"/>
     </row>
     <row r="90">
-      <c r="B90" s="2" t="n"/>
-      <c r="C90" s="2" t="n"/>
+      <c r="B90" s="3" t="n"/>
+      <c r="C90" s="3" t="n"/>
     </row>
     <row r="91">
-      <c r="B91" s="2" t="n"/>
-      <c r="C91" s="2" t="n"/>
+      <c r="B91" s="3" t="n"/>
+      <c r="C91" s="3" t="n"/>
     </row>
     <row r="92">
-      <c r="B92" s="2" t="n"/>
-      <c r="C92" s="2" t="n"/>
+      <c r="B92" s="3" t="n"/>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
-      <c r="B93" s="2" t="n"/>
-      <c r="C93" s="2" t="n"/>
+      <c r="B93" s="3" t="n"/>
+      <c r="C93" s="3" t="n"/>
     </row>
     <row r="94">
-      <c r="B94" s="2" t="n"/>
-      <c r="C94" s="2" t="n"/>
+      <c r="B94" s="3" t="n"/>
+      <c r="C94" s="3" t="n"/>
     </row>
     <row r="95">
-      <c r="B95" s="2" t="n"/>
-      <c r="C95" s="2" t="n"/>
+      <c r="B95" s="3" t="n"/>
+      <c r="C95" s="3" t="n"/>
     </row>
     <row r="96">
-      <c r="B96" s="2" t="n"/>
-      <c r="C96" s="2" t="n"/>
+      <c r="B96" s="3" t="n"/>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
-      <c r="B97" s="2" t="n"/>
-      <c r="C97" s="2" t="n"/>
+      <c r="B97" s="3" t="n"/>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
-      <c r="B98" s="2" t="n"/>
-      <c r="C98" s="2" t="n"/>
+      <c r="B98" s="3" t="n"/>
+      <c r="C98" s="3" t="n"/>
     </row>
     <row r="99">
-      <c r="B99" s="2" t="n"/>
-      <c r="C99" s="2" t="n"/>
+      <c r="B99" s="3" t="n"/>
+      <c r="C99" s="3" t="n"/>
     </row>
     <row r="100">
-      <c r="B100" s="2" t="n"/>
-      <c r="C100" s="2" t="n"/>
+      <c r="B100" s="3" t="n"/>
+      <c r="C100" s="3" t="n"/>
     </row>
     <row r="101">
-      <c r="B101" s="2" t="n"/>
-      <c r="C101" s="2" t="n"/>
+      <c r="B101" s="3" t="n"/>
+      <c r="C101" s="3" t="n"/>
     </row>
     <row r="102">
-      <c r="B102" s="2" t="n"/>
-      <c r="C102" s="2" t="n"/>
+      <c r="B102" s="3" t="n"/>
+      <c r="C102" s="3" t="n"/>
     </row>
     <row r="103">
-      <c r="B103" s="2" t="n"/>
-      <c r="C103" s="2" t="n"/>
+      <c r="B103" s="3" t="n"/>
+      <c r="C103" s="3" t="n"/>
     </row>
     <row r="104">
-      <c r="B104" s="2" t="n"/>
-      <c r="C104" s="2" t="n"/>
+      <c r="B104" s="3" t="n"/>
+      <c r="C104" s="3" t="n"/>
     </row>
     <row r="105">
-      <c r="B105" s="2" t="n"/>
-      <c r="C105" s="2" t="n"/>
+      <c r="B105" s="3" t="n"/>
+      <c r="C105" s="3" t="n"/>
     </row>
     <row r="106">
-      <c r="B106" s="2" t="n"/>
-      <c r="C106" s="2" t="n"/>
+      <c r="B106" s="3" t="n"/>
+      <c r="C106" s="3" t="n"/>
     </row>
     <row r="107">
-      <c r="B107" s="2" t="n"/>
-      <c r="C107" s="2" t="n"/>
+      <c r="B107" s="3" t="n"/>
+      <c r="C107" s="3" t="n"/>
     </row>
     <row r="108">
-      <c r="B108" s="2" t="n"/>
-      <c r="C108" s="2" t="n"/>
+      <c r="B108" s="3" t="n"/>
+      <c r="C108" s="3" t="n"/>
     </row>
     <row r="109">
-      <c r="B109" s="2" t="n"/>
-      <c r="C109" s="2" t="n"/>
+      <c r="B109" s="3" t="n"/>
+      <c r="C109" s="3" t="n"/>
     </row>
     <row r="110">
-      <c r="B110" s="2" t="n"/>
-      <c r="C110" s="2" t="n"/>
+      <c r="B110" s="3" t="n"/>
+      <c r="C110" s="3" t="n"/>
     </row>
     <row r="111">
-      <c r="B111" s="2" t="n"/>
-      <c r="C111" s="2" t="n"/>
+      <c r="B111" s="3" t="n"/>
+      <c r="C111" s="3" t="n"/>
     </row>
     <row r="112">
-      <c r="B112" s="2" t="n"/>
-      <c r="C112" s="2" t="n"/>
+      <c r="B112" s="3" t="n"/>
+      <c r="C112" s="3" t="n"/>
     </row>
     <row r="113">
-      <c r="B113" s="2" t="n"/>
-      <c r="C113" s="2" t="n"/>
+      <c r="B113" s="3" t="n"/>
+      <c r="C113" s="3" t="n"/>
     </row>
     <row r="114">
-      <c r="B114" s="2" t="n"/>
-      <c r="C114" s="2" t="n"/>
+      <c r="B114" s="3" t="n"/>
+      <c r="C114" s="3" t="n"/>
     </row>
     <row r="115">
-      <c r="B115" s="2" t="n"/>
-      <c r="C115" s="2" t="n"/>
+      <c r="B115" s="3" t="n"/>
+      <c r="C115" s="3" t="n"/>
     </row>
     <row r="116">
-      <c r="B116" s="2" t="n"/>
-      <c r="C116" s="2" t="n"/>
+      <c r="B116" s="3" t="n"/>
+      <c r="C116" s="3" t="n"/>
     </row>
     <row r="117">
-      <c r="B117" s="2" t="n"/>
-      <c r="C117" s="2" t="n"/>
+      <c r="B117" s="3" t="n"/>
+      <c r="C117" s="3" t="n"/>
     </row>
     <row r="118">
-      <c r="B118" s="2" t="n"/>
-      <c r="C118" s="2" t="n"/>
+      <c r="B118" s="3" t="n"/>
+      <c r="C118" s="3" t="n"/>
     </row>
     <row r="119">
-      <c r="B119" s="2" t="n"/>
-      <c r="C119" s="2" t="n"/>
+      <c r="B119" s="3" t="n"/>
+      <c r="C119" s="3" t="n"/>
     </row>
     <row r="120">
-      <c r="B120" s="2" t="n"/>
-      <c r="C120" s="2" t="n"/>
+      <c r="B120" s="3" t="n"/>
+      <c r="C120" s="3" t="n"/>
     </row>
     <row r="121">
-      <c r="B121" s="2" t="n"/>
-      <c r="C121" s="2" t="n"/>
+      <c r="B121" s="3" t="n"/>
+      <c r="C121" s="3" t="n"/>
     </row>
     <row r="122">
-      <c r="B122" s="2" t="n"/>
-      <c r="C122" s="2" t="n"/>
+      <c r="B122" s="3" t="n"/>
+      <c r="C122" s="3" t="n"/>
     </row>
     <row r="123">
-      <c r="B123" s="2" t="n"/>
-      <c r="C123" s="2" t="n"/>
+      <c r="B123" s="3" t="n"/>
+      <c r="C123" s="3" t="n"/>
     </row>
     <row r="124">
-      <c r="B124" s="2" t="n"/>
-      <c r="C124" s="2" t="n"/>
+      <c r="B124" s="3" t="n"/>
+      <c r="C124" s="3" t="n"/>
     </row>
     <row r="125">
-      <c r="B125" s="2" t="n"/>
-      <c r="C125" s="2" t="n"/>
+      <c r="B125" s="3" t="n"/>
+      <c r="C125" s="3" t="n"/>
     </row>
     <row r="126">
-      <c r="B126" s="2" t="n"/>
-      <c r="C126" s="2" t="n"/>
+      <c r="B126" s="3" t="n"/>
+      <c r="C126" s="3" t="n"/>
     </row>
     <row r="127">
-      <c r="B127" s="2" t="n"/>
-      <c r="C127" s="2" t="n"/>
+      <c r="B127" s="3" t="n"/>
+      <c r="C127" s="3" t="n"/>
     </row>
     <row r="128">
-      <c r="B128" s="2" t="n"/>
-      <c r="C128" s="2" t="n"/>
+      <c r="B128" s="3" t="n"/>
+      <c r="C128" s="3" t="n"/>
     </row>
     <row r="129">
-      <c r="B129" s="2" t="n"/>
-      <c r="C129" s="2" t="n"/>
+      <c r="B129" s="3" t="n"/>
+      <c r="C129" s="3" t="n"/>
     </row>
     <row r="130">
-      <c r="B130" s="2" t="n"/>
-      <c r="C130" s="2" t="n"/>
+      <c r="B130" s="3" t="n"/>
+      <c r="C130" s="3" t="n"/>
     </row>
     <row r="131">
-      <c r="B131" s="2" t="n"/>
-      <c r="C131" s="2" t="n"/>
+      <c r="B131" s="3" t="n"/>
+      <c r="C131" s="3" t="n"/>
     </row>
     <row r="132">
-      <c r="B132" s="2" t="n"/>
-      <c r="C132" s="2" t="n"/>
+      <c r="B132" s="3" t="n"/>
+      <c r="C132" s="3" t="n"/>
     </row>
     <row r="133">
-      <c r="B133" s="2" t="n"/>
-      <c r="C133" s="2" t="n"/>
+      <c r="B133" s="3" t="n"/>
+      <c r="C133" s="3" t="n"/>
     </row>
     <row r="134">
-      <c r="B134" s="2" t="n"/>
-      <c r="C134" s="2" t="n"/>
+      <c r="B134" s="3" t="n"/>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
-      <c r="B135" s="2" t="n"/>
-      <c r="C135" s="2" t="n"/>
+      <c r="B135" s="3" t="n"/>
+      <c r="C135" s="3" t="n"/>
     </row>
     <row r="136">
-      <c r="B136" s="2" t="n"/>
-      <c r="C136" s="2" t="n"/>
+      <c r="B136" s="3" t="n"/>
+      <c r="C136" s="3" t="n"/>
     </row>
     <row r="137">
-      <c r="B137" s="2" t="n"/>
-      <c r="C137" s="2" t="n"/>
+      <c r="B137" s="3" t="n"/>
+      <c r="C137" s="3" t="n"/>
     </row>
     <row r="138">
-      <c r="B138" s="2" t="n"/>
-      <c r="C138" s="2" t="n"/>
+      <c r="B138" s="3" t="n"/>
+      <c r="C138" s="3" t="n"/>
     </row>
     <row r="139">
-      <c r="B139" s="2" t="n"/>
-      <c r="C139" s="2" t="n"/>
+      <c r="B139" s="3" t="n"/>
+      <c r="C139" s="3" t="n"/>
     </row>
     <row r="140">
-      <c r="B140" s="2" t="n"/>
-      <c r="C140" s="2" t="n"/>
+      <c r="B140" s="3" t="n"/>
+      <c r="C140" s="3" t="n"/>
     </row>
     <row r="141">
-      <c r="B141" s="2" t="n"/>
-      <c r="C141" s="2" t="n"/>
+      <c r="B141" s="3" t="n"/>
+      <c r="C141" s="3" t="n"/>
     </row>
     <row r="142">
-      <c r="B142" s="2" t="n"/>
-      <c r="C142" s="2" t="n"/>
+      <c r="B142" s="3" t="n"/>
+      <c r="C142" s="3" t="n"/>
     </row>
     <row r="143">
-      <c r="B143" s="2" t="n"/>
-      <c r="C143" s="2" t="n"/>
+      <c r="B143" s="3" t="n"/>
+      <c r="C143" s="3" t="n"/>
     </row>
     <row r="144">
-      <c r="B144" s="2" t="n"/>
-      <c r="C144" s="2" t="n"/>
+      <c r="B144" s="3" t="n"/>
+      <c r="C144" s="3" t="n"/>
     </row>
     <row r="145">
-      <c r="B145" s="2" t="n"/>
-      <c r="C145" s="2" t="n"/>
+      <c r="B145" s="3" t="n"/>
+      <c r="C145" s="3" t="n"/>
     </row>
     <row r="146">
-      <c r="B146" s="2" t="n"/>
-      <c r="C146" s="2" t="n"/>
+      <c r="B146" s="3" t="n"/>
+      <c r="C146" s="3" t="n"/>
     </row>
     <row r="147">
-      <c r="B147" s="2" t="n"/>
-      <c r="C147" s="2" t="n"/>
+      <c r="B147" s="3" t="n"/>
+      <c r="C147" s="3" t="n"/>
     </row>
     <row r="148">
-      <c r="B148" s="2" t="n"/>
-      <c r="C148" s="2" t="n"/>
+      <c r="B148" s="3" t="n"/>
+      <c r="C148" s="3" t="n"/>
     </row>
     <row r="149">
-      <c r="B149" s="2" t="n"/>
-      <c r="C149" s="2" t="n"/>
+      <c r="B149" s="3" t="n"/>
+      <c r="C149" s="3" t="n"/>
     </row>
     <row r="150">
-      <c r="B150" s="2" t="n"/>
-      <c r="C150" s="2" t="n"/>
+      <c r="B150" s="3" t="n"/>
+      <c r="C150" s="3" t="n"/>
     </row>
     <row r="151">
-      <c r="B151" s="2" t="n"/>
-      <c r="C151" s="2" t="n"/>
+      <c r="B151" s="3" t="n"/>
+      <c r="C151" s="3" t="n"/>
     </row>
     <row r="152">
-      <c r="B152" s="2" t="n"/>
-      <c r="C152" s="2" t="n"/>
+      <c r="B152" s="3" t="n"/>
+      <c r="C152" s="3" t="n"/>
     </row>
     <row r="153">
-      <c r="B153" s="2" t="n"/>
-      <c r="C153" s="2" t="n"/>
+      <c r="B153" s="3" t="n"/>
+      <c r="C153" s="3" t="n"/>
     </row>
     <row r="154">
-      <c r="B154" s="2" t="n"/>
-      <c r="C154" s="2" t="n"/>
+      <c r="B154" s="3" t="n"/>
+      <c r="C154" s="3" t="n"/>
     </row>
     <row r="155">
-      <c r="B155" s="2" t="n"/>
-      <c r="C155" s="2" t="n"/>
+      <c r="B155" s="3" t="n"/>
+      <c r="C155" s="3" t="n"/>
     </row>
     <row r="156">
-      <c r="B156" s="2" t="n"/>
-      <c r="C156" s="2" t="n"/>
+      <c r="B156" s="3" t="n"/>
+      <c r="C156" s="3" t="n"/>
     </row>
     <row r="157">
-      <c r="B157" s="2" t="n"/>
-      <c r="C157" s="2" t="n"/>
+      <c r="B157" s="3" t="n"/>
+      <c r="C157" s="3" t="n"/>
     </row>
     <row r="158">
-      <c r="B158" s="2" t="n"/>
-      <c r="C158" s="2" t="n"/>
+      <c r="B158" s="3" t="n"/>
+      <c r="C158" s="3" t="n"/>
     </row>
     <row r="159">
-      <c r="B159" s="2" t="n"/>
-      <c r="C159" s="2" t="n"/>
+      <c r="B159" s="3" t="n"/>
+      <c r="C159" s="3" t="n"/>
     </row>
     <row r="160">
-      <c r="B160" s="2" t="n"/>
-      <c r="C160" s="2" t="n"/>
+      <c r="B160" s="3" t="n"/>
+      <c r="C160" s="3" t="n"/>
     </row>
     <row r="161">
-      <c r="B161" s="2" t="n"/>
-      <c r="C161" s="2" t="n"/>
+      <c r="B161" s="3" t="n"/>
+      <c r="C161" s="3" t="n"/>
     </row>
     <row r="162">
-      <c r="B162" s="2" t="n"/>
-      <c r="C162" s="2" t="n"/>
+      <c r="B162" s="3" t="n"/>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
-      <c r="B163" s="2" t="n"/>
-      <c r="C163" s="2" t="n"/>
+      <c r="B163" s="3" t="n"/>
+      <c r="C163" s="3" t="n"/>
     </row>
     <row r="164">
-      <c r="B164" s="2" t="n"/>
-      <c r="C164" s="2" t="n"/>
+      <c r="B164" s="3" t="n"/>
+      <c r="C164" s="3" t="n"/>
     </row>
     <row r="165">
-      <c r="B165" s="2" t="n"/>
-      <c r="C165" s="2" t="n"/>
+      <c r="B165" s="3" t="n"/>
+      <c r="C165" s="3" t="n"/>
     </row>
     <row r="166">
-      <c r="B166" s="2" t="n"/>
-      <c r="C166" s="2" t="n"/>
+      <c r="B166" s="3" t="n"/>
+      <c r="C166" s="3" t="n"/>
     </row>
     <row r="167">
-      <c r="B167" s="2" t="n"/>
-      <c r="C167" s="2" t="n"/>
+      <c r="B167" s="3" t="n"/>
+      <c r="C167" s="3" t="n"/>
     </row>
     <row r="168">
-      <c r="B168" s="2" t="n"/>
-      <c r="C168" s="2" t="n"/>
+      <c r="B168" s="3" t="n"/>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
-      <c r="B169" s="2" t="n"/>
-      <c r="C169" s="2" t="n"/>
+      <c r="B169" s="3" t="n"/>
+      <c r="C169" s="3" t="n"/>
     </row>
     <row r="170">
-      <c r="B170" s="2" t="n"/>
-      <c r="C170" s="2" t="n"/>
+      <c r="B170" s="3" t="n"/>
+      <c r="C170" s="3" t="n"/>
     </row>
     <row r="171">
-      <c r="B171" s="2" t="n"/>
-      <c r="C171" s="2" t="n"/>
+      <c r="B171" s="3" t="n"/>
+      <c r="C171" s="3" t="n"/>
     </row>
     <row r="172">
-      <c r="B172" s="2" t="n"/>
-      <c r="C172" s="2" t="n"/>
+      <c r="B172" s="3" t="n"/>
+      <c r="C172" s="3" t="n"/>
     </row>
     <row r="173">
-      <c r="B173" s="2" t="n"/>
-      <c r="C173" s="2" t="n"/>
+      <c r="B173" s="3" t="n"/>
+      <c r="C173" s="3" t="n"/>
     </row>
     <row r="174">
-      <c r="B174" s="2" t="n"/>
-      <c r="C174" s="2" t="n"/>
+      <c r="B174" s="3" t="n"/>
+      <c r="C174" s="3" t="n"/>
     </row>
     <row r="175">
-      <c r="B175" s="2" t="n"/>
-      <c r="C175" s="2" t="n"/>
+      <c r="B175" s="3" t="n"/>
+      <c r="C175" s="3" t="n"/>
     </row>
     <row r="176">
-      <c r="B176" s="2" t="n"/>
-      <c r="C176" s="2" t="n"/>
+      <c r="B176" s="3" t="n"/>
+      <c r="C176" s="3" t="n"/>
     </row>
     <row r="177">
-      <c r="B177" s="2" t="n"/>
-      <c r="C177" s="2" t="n"/>
+      <c r="B177" s="3" t="n"/>
+      <c r="C177" s="3" t="n"/>
     </row>
     <row r="178">
-      <c r="B178" s="2" t="n"/>
-      <c r="C178" s="2" t="n"/>
+      <c r="B178" s="3" t="n"/>
+      <c r="C178" s="3" t="n"/>
     </row>
     <row r="179">
-      <c r="B179" s="2" t="n"/>
-      <c r="C179" s="2" t="n"/>
+      <c r="B179" s="3" t="n"/>
+      <c r="C179" s="3" t="n"/>
     </row>
     <row r="180">
-      <c r="B180" s="2" t="n"/>
-      <c r="C180" s="2" t="n"/>
+      <c r="B180" s="3" t="n"/>
+      <c r="C180" s="3" t="n"/>
     </row>
     <row r="181">
-      <c r="B181" s="2" t="n"/>
-      <c r="C181" s="2" t="n"/>
+      <c r="B181" s="3" t="n"/>
+      <c r="C181" s="3" t="n"/>
     </row>
     <row r="182">
-      <c r="B182" s="2" t="n"/>
-      <c r="C182" s="2" t="n"/>
+      <c r="B182" s="3" t="n"/>
+      <c r="C182" s="3" t="n"/>
     </row>
     <row r="183">
-      <c r="B183" s="2" t="n"/>
-      <c r="C183" s="2" t="n"/>
+      <c r="B183" s="3" t="n"/>
+      <c r="C183" s="3" t="n"/>
     </row>
     <row r="184">
-      <c r="B184" s="2" t="n"/>
-      <c r="C184" s="2" t="n"/>
+      <c r="B184" s="3" t="n"/>
+      <c r="C184" s="3" t="n"/>
     </row>
     <row r="185">
-      <c r="B185" s="2" t="n"/>
-      <c r="C185" s="2" t="n"/>
+      <c r="B185" s="3" t="n"/>
+      <c r="C185" s="3" t="n"/>
     </row>
     <row r="186">
-      <c r="B186" s="2" t="n"/>
-      <c r="C186" s="2" t="n"/>
+      <c r="B186" s="3" t="n"/>
+      <c r="C186" s="3" t="n"/>
     </row>
     <row r="187">
-      <c r="B187" s="2" t="n"/>
-      <c r="C187" s="2" t="n"/>
+      <c r="B187" s="3" t="n"/>
+      <c r="C187" s="3" t="n"/>
     </row>
     <row r="188">
-      <c r="B188" s="2" t="n"/>
-      <c r="C188" s="2" t="n"/>
+      <c r="B188" s="3" t="n"/>
+      <c r="C188" s="3" t="n"/>
     </row>
     <row r="189">
-      <c r="B189" s="2" t="n"/>
-      <c r="C189" s="2" t="n"/>
+      <c r="B189" s="3" t="n"/>
+      <c r="C189" s="3" t="n"/>
     </row>
     <row r="190">
-      <c r="B190" s="2" t="n"/>
-      <c r="C190" s="2" t="n"/>
+      <c r="B190" s="3" t="n"/>
+      <c r="C190" s="3" t="n"/>
     </row>
     <row r="191">
-      <c r="B191" s="2" t="n"/>
-      <c r="C191" s="2" t="n"/>
+      <c r="B191" s="3" t="n"/>
+      <c r="C191" s="3" t="n"/>
     </row>
     <row r="192">
-      <c r="B192" s="2" t="n"/>
-      <c r="C192" s="2" t="n"/>
+      <c r="B192" s="3" t="n"/>
+      <c r="C192" s="3" t="n"/>
     </row>
     <row r="193">
-      <c r="B193" s="2" t="n"/>
-      <c r="C193" s="2" t="n"/>
+      <c r="B193" s="3" t="n"/>
+      <c r="C193" s="3" t="n"/>
     </row>
     <row r="194">
-      <c r="B194" s="2" t="n"/>
-      <c r="C194" s="2" t="n"/>
+      <c r="B194" s="3" t="n"/>
+      <c r="C194" s="3" t="n"/>
     </row>
     <row r="195">
-      <c r="B195" s="2" t="n"/>
-      <c r="C195" s="2" t="n"/>
+      <c r="B195" s="3" t="n"/>
+      <c r="C195" s="3" t="n"/>
     </row>
     <row r="196">
-      <c r="B196" s="2" t="n"/>
-      <c r="C196" s="2" t="n"/>
+      <c r="B196" s="3" t="n"/>
+      <c r="C196" s="3" t="n"/>
     </row>
     <row r="197">
-      <c r="B197" s="2" t="n"/>
-      <c r="C197" s="2" t="n"/>
+      <c r="B197" s="3" t="n"/>
+      <c r="C197" s="3" t="n"/>
     </row>
     <row r="198">
-      <c r="B198" s="2" t="n"/>
-      <c r="C198" s="2" t="n"/>
+      <c r="B198" s="3" t="n"/>
+      <c r="C198" s="3" t="n"/>
     </row>
     <row r="199">
-      <c r="B199" s="2" t="n"/>
-      <c r="C199" s="2" t="n"/>
+      <c r="B199" s="3" t="n"/>
+      <c r="C199" s="3" t="n"/>
     </row>
     <row r="200">
-      <c r="B200" s="2" t="n"/>
-      <c r="C200" s="2" t="n"/>
+      <c r="B200" s="3" t="n"/>
+      <c r="C200" s="3" t="n"/>
     </row>
     <row r="201">
-      <c r="B201" s="2" t="n"/>
-      <c r="C201" s="2" t="n"/>
+      <c r="B201" s="3" t="n"/>
+      <c r="C201" s="3" t="n"/>
     </row>
     <row r="202">
-      <c r="B202" s="2" t="n"/>
-      <c r="C202" s="2" t="n"/>
+      <c r="B202" s="3" t="n"/>
+      <c r="C202" s="3" t="n"/>
     </row>
     <row r="203">
-      <c r="B203" s="2" t="n"/>
-      <c r="C203" s="2" t="n"/>
+      <c r="B203" s="3" t="n"/>
+      <c r="C203" s="3" t="n"/>
     </row>
     <row r="204">
-      <c r="B204" s="2" t="n"/>
-      <c r="C204" s="2" t="n"/>
+      <c r="B204" s="3" t="n"/>
+      <c r="C204" s="3" t="n"/>
     </row>
     <row r="205">
-      <c r="B205" s="2" t="n"/>
-      <c r="C205" s="2" t="n"/>
+      <c r="B205" s="3" t="n"/>
+      <c r="C205" s="3" t="n"/>
     </row>
     <row r="206">
-      <c r="B206" s="2" t="n"/>
-      <c r="C206" s="2" t="n"/>
+      <c r="B206" s="3" t="n"/>
+      <c r="C206" s="3" t="n"/>
     </row>
     <row r="207">
-      <c r="B207" s="2" t="n"/>
-      <c r="C207" s="2" t="n"/>
+      <c r="B207" s="3" t="n"/>
+      <c r="C207" s="3" t="n"/>
     </row>
     <row r="208">
-      <c r="B208" s="2" t="n"/>
-      <c r="C208" s="2" t="n"/>
+      <c r="B208" s="3" t="n"/>
+      <c r="C208" s="3" t="n"/>
     </row>
     <row r="209">
-      <c r="B209" s="2" t="n"/>
-      <c r="C209" s="2" t="n"/>
+      <c r="B209" s="3" t="n"/>
+      <c r="C209" s="3" t="n"/>
     </row>
     <row r="210">
-      <c r="B210" s="2" t="n"/>
-      <c r="C210" s="2" t="n"/>
+      <c r="B210" s="3" t="n"/>
+      <c r="C210" s="3" t="n"/>
     </row>
     <row r="211">
-      <c r="B211" s="2" t="n"/>
-      <c r="C211" s="2" t="n"/>
+      <c r="B211" s="3" t="n"/>
+      <c r="C211" s="3" t="n"/>
     </row>
     <row r="212">
-      <c r="B212" s="2" t="n"/>
-      <c r="C212" s="2" t="n"/>
+      <c r="B212" s="3" t="n"/>
+      <c r="C212" s="3" t="n"/>
     </row>
     <row r="213">
-      <c r="B213" s="2" t="n"/>
-      <c r="C213" s="2" t="n"/>
+      <c r="B213" s="3" t="n"/>
+      <c r="C213" s="3" t="n"/>
     </row>
     <row r="214">
-      <c r="B214" s="2" t="n"/>
-      <c r="C214" s="2" t="n"/>
+      <c r="B214" s="3" t="n"/>
+      <c r="C214" s="3" t="n"/>
     </row>
     <row r="215">
-      <c r="B215" s="2" t="n"/>
-      <c r="C215" s="2" t="n"/>
+      <c r="B215" s="3" t="n"/>
+      <c r="C215" s="3" t="n"/>
     </row>
     <row r="216">
-      <c r="B216" s="2" t="n"/>
-      <c r="C216" s="2" t="n"/>
+      <c r="B216" s="3" t="n"/>
+      <c r="C216" s="3" t="n"/>
     </row>
     <row r="217">
-      <c r="B217" s="2" t="n"/>
-      <c r="C217" s="2" t="n"/>
+      <c r="B217" s="3" t="n"/>
+      <c r="C217" s="3" t="n"/>
     </row>
     <row r="218">
-      <c r="B218" s="2" t="n"/>
-      <c r="C218" s="2" t="n"/>
+      <c r="B218" s="3" t="n"/>
+      <c r="C218" s="3" t="n"/>
     </row>
     <row r="219">
-      <c r="B219" s="2" t="n"/>
-      <c r="C219" s="2" t="n"/>
+      <c r="B219" s="3" t="n"/>
+      <c r="C219" s="3" t="n"/>
     </row>
     <row r="220">
-      <c r="B220" s="2" t="n"/>
-      <c r="C220" s="2" t="n"/>
+      <c r="B220" s="3" t="n"/>
+      <c r="C220" s="3" t="n"/>
     </row>
     <row r="221">
-      <c r="B221" s="2" t="n"/>
-      <c r="C221" s="2" t="n"/>
+      <c r="B221" s="3" t="n"/>
+      <c r="C221" s="3" t="n"/>
     </row>
     <row r="222">
-      <c r="B222" s="2" t="n"/>
-      <c r="C222" s="2" t="n"/>
+      <c r="B222" s="3" t="n"/>
+      <c r="C222" s="3" t="n"/>
     </row>
     <row r="223">
-      <c r="B223" s="2" t="n"/>
-      <c r="C223" s="2" t="n"/>
+      <c r="B223" s="3" t="n"/>
+      <c r="C223" s="3" t="n"/>
     </row>
     <row r="224">
-      <c r="B224" s="2" t="n"/>
-      <c r="C224" s="2" t="n"/>
+      <c r="B224" s="3" t="n"/>
+      <c r="C224" s="3" t="n"/>
     </row>
     <row r="225">
-      <c r="B225" s="2" t="n"/>
-      <c r="C225" s="2" t="n"/>
+      <c r="B225" s="3" t="n"/>
+      <c r="C225" s="3" t="n"/>
     </row>
     <row r="226">
-      <c r="B226" s="2" t="n"/>
-      <c r="C226" s="2" t="n"/>
+      <c r="B226" s="3" t="n"/>
+      <c r="C226" s="3" t="n"/>
     </row>
     <row r="227">
-      <c r="B227" s="2" t="n"/>
-      <c r="C227" s="2" t="n"/>
+      <c r="B227" s="3" t="n"/>
+      <c r="C227" s="3" t="n"/>
     </row>
     <row r="228">
-      <c r="B228" s="2" t="n"/>
-      <c r="C228" s="2" t="n"/>
+      <c r="B228" s="3" t="n"/>
+      <c r="C228" s="3" t="n"/>
     </row>
     <row r="229">
-      <c r="B229" s="2" t="n"/>
-      <c r="C229" s="2" t="n"/>
+      <c r="B229" s="3" t="n"/>
+      <c r="C229" s="3" t="n"/>
     </row>
     <row r="230">
-      <c r="B230" s="2" t="n"/>
-      <c r="C230" s="2" t="n"/>
+      <c r="B230" s="3" t="n"/>
+      <c r="C230" s="3" t="n"/>
     </row>
     <row r="231">
-      <c r="B231" s="2" t="n"/>
-      <c r="C231" s="2" t="n"/>
+      <c r="B231" s="3" t="n"/>
+      <c r="C231" s="3" t="n"/>
     </row>
     <row r="232">
-      <c r="B232" s="2" t="n"/>
-      <c r="C232" s="2" t="n"/>
+      <c r="B232" s="3" t="n"/>
+      <c r="C232" s="3" t="n"/>
     </row>
     <row r="233">
-      <c r="B233" s="2" t="n"/>
-      <c r="C233" s="2" t="n"/>
+      <c r="B233" s="3" t="n"/>
+      <c r="C233" s="3" t="n"/>
     </row>
     <row r="234">
-      <c r="B234" s="2" t="n"/>
-      <c r="C234" s="2" t="n"/>
+      <c r="B234" s="3" t="n"/>
+      <c r="C234" s="3" t="n"/>
     </row>
     <row r="235">
-      <c r="B235" s="2" t="n"/>
-      <c r="C235" s="2" t="n"/>
+      <c r="B235" s="3" t="n"/>
+      <c r="C235" s="3" t="n"/>
     </row>
     <row r="236">
-      <c r="B236" s="2" t="n"/>
-      <c r="C236" s="2" t="n"/>
+      <c r="B236" s="3" t="n"/>
+      <c r="C236" s="3" t="n"/>
     </row>
     <row r="237">
-      <c r="B237" s="2" t="n"/>
-      <c r="C237" s="2" t="n"/>
+      <c r="B237" s="3" t="n"/>
+      <c r="C237" s="3" t="n"/>
     </row>
     <row r="238">
-      <c r="B238" s="2" t="n"/>
-      <c r="C238" s="2" t="n"/>
+      <c r="B238" s="3" t="n"/>
+      <c r="C238" s="3" t="n"/>
     </row>
     <row r="239">
-      <c r="B239" s="2" t="n"/>
-      <c r="C239" s="2" t="n"/>
+      <c r="B239" s="3" t="n"/>
+      <c r="C239" s="3" t="n"/>
     </row>
     <row r="240">
-      <c r="B240" s="2" t="n"/>
-      <c r="C240" s="2" t="n"/>
+      <c r="B240" s="3" t="n"/>
+      <c r="C240" s="3" t="n"/>
     </row>
     <row r="241">
-      <c r="B241" s="2" t="n"/>
-      <c r="C241" s="2" t="n"/>
+      <c r="B241" s="3" t="n"/>
+      <c r="C241" s="3" t="n"/>
     </row>
     <row r="242">
-      <c r="B242" s="2" t="n"/>
-      <c r="C242" s="2" t="n"/>
+      <c r="B242" s="3" t="n"/>
+      <c r="C242" s="3" t="n"/>
     </row>
     <row r="243">
-      <c r="B243" s="2" t="n"/>
-      <c r="C243" s="2" t="n"/>
+      <c r="B243" s="3" t="n"/>
+      <c r="C243" s="3" t="n"/>
     </row>
     <row r="244">
-      <c r="B244" s="2" t="n"/>
-      <c r="C244" s="2" t="n"/>
+      <c r="B244" s="3" t="n"/>
+      <c r="C244" s="3" t="n"/>
     </row>
     <row r="245">
-      <c r="B245" s="2" t="n"/>
-      <c r="C245" s="2" t="n"/>
+      <c r="B245" s="3" t="n"/>
+      <c r="C245" s="3" t="n"/>
     </row>
     <row r="246">
-      <c r="B246" s="2" t="n"/>
-      <c r="C246" s="2" t="n"/>
+      <c r="B246" s="3" t="n"/>
+      <c r="C246" s="3" t="n"/>
     </row>
     <row r="247">
-      <c r="B247" s="2" t="n"/>
-      <c r="C247" s="2" t="n"/>
+      <c r="B247" s="3" t="n"/>
+      <c r="C247" s="3" t="n"/>
     </row>
     <row r="248">
-      <c r="B248" s="2" t="n"/>
-      <c r="C248" s="2" t="n"/>
+      <c r="B248" s="3" t="n"/>
+      <c r="C248" s="3" t="n"/>
     </row>
     <row r="249">
-      <c r="B249" s="2" t="n"/>
-      <c r="C249" s="2" t="n"/>
+      <c r="B249" s="3" t="n"/>
+      <c r="C249" s="3" t="n"/>
     </row>
     <row r="250">
-      <c r="B250" s="2" t="n"/>
-      <c r="C250" s="2" t="n"/>
+      <c r="B250" s="3" t="n"/>
+      <c r="C250" s="3" t="n"/>
     </row>
     <row r="251">
-      <c r="B251" s="2" t="n"/>
-      <c r="C251" s="2" t="n"/>
+      <c r="B251" s="3" t="n"/>
+      <c r="C251" s="3" t="n"/>
     </row>
     <row r="252">
-      <c r="B252" s="2" t="n"/>
-      <c r="C252" s="2" t="n"/>
+      <c r="B252" s="3" t="n"/>
+      <c r="C252" s="3" t="n"/>
     </row>
     <row r="253">
-      <c r="B253" s="2" t="n"/>
-      <c r="C253" s="2" t="n"/>
+      <c r="B253" s="3" t="n"/>
+      <c r="C253" s="3" t="n"/>
     </row>
     <row r="254">
-      <c r="B254" s="2" t="n"/>
-      <c r="C254" s="2" t="n"/>
+      <c r="B254" s="3" t="n"/>
+      <c r="C254" s="3" t="n"/>
     </row>
     <row r="255">
-      <c r="B255" s="2" t="n"/>
-      <c r="C255" s="2" t="n"/>
+      <c r="B255" s="3" t="n"/>
+      <c r="C255" s="3" t="n"/>
     </row>
     <row r="256">
-      <c r="B256" s="2" t="n"/>
-      <c r="C256" s="2" t="n"/>
+      <c r="B256" s="3" t="n"/>
+      <c r="C256" s="3" t="n"/>
     </row>
     <row r="257">
-      <c r="B257" s="2" t="n"/>
-      <c r="C257" s="2" t="n"/>
+      <c r="B257" s="3" t="n"/>
+      <c r="C257" s="3" t="n"/>
     </row>
     <row r="258">
-      <c r="B258" s="2" t="n"/>
-      <c r="C258" s="2" t="n"/>
+      <c r="B258" s="3" t="n"/>
+      <c r="C258" s="3" t="n"/>
     </row>
     <row r="259">
-      <c r="B259" s="2" t="n"/>
-      <c r="C259" s="2" t="n"/>
+      <c r="B259" s="3" t="n"/>
+      <c r="C259" s="3" t="n"/>
     </row>
     <row r="260">
-      <c r="B260" s="2" t="n"/>
-      <c r="C260" s="2" t="n"/>
+      <c r="B260" s="3" t="n"/>
+      <c r="C260" s="3" t="n"/>
     </row>
     <row r="261">
-      <c r="B261" s="2" t="n"/>
-      <c r="C261" s="2" t="n"/>
+      <c r="B261" s="3" t="n"/>
+      <c r="C261" s="3" t="n"/>
     </row>
     <row r="262">
-      <c r="B262" s="2" t="n"/>
-      <c r="C262" s="2" t="n"/>
+      <c r="B262" s="3" t="n"/>
+      <c r="C262" s="3" t="n"/>
     </row>
     <row r="263">
-      <c r="B263" s="2" t="n"/>
-      <c r="C263" s="2" t="n"/>
+      <c r="B263" s="3" t="n"/>
+      <c r="C263" s="3" t="n"/>
     </row>
     <row r="264">
-      <c r="B264" s="2" t="n"/>
-      <c r="C264" s="2" t="n"/>
+      <c r="B264" s="3" t="n"/>
+      <c r="C264" s="3" t="n"/>
     </row>
     <row r="265">
-      <c r="B265" s="2" t="n"/>
-      <c r="C265" s="2" t="n"/>
+      <c r="B265" s="3" t="n"/>
+      <c r="C265" s="3" t="n"/>
     </row>
     <row r="266">
-      <c r="B266" s="2" t="n"/>
-      <c r="C266" s="2" t="n"/>
+      <c r="B266" s="3" t="n"/>
+      <c r="C266" s="3" t="n"/>
     </row>
     <row r="267">
-      <c r="B267" s="2" t="n"/>
-      <c r="C267" s="2" t="n"/>
+      <c r="B267" s="3" t="n"/>
+      <c r="C267" s="3" t="n"/>
     </row>
     <row r="268">
-      <c r="B268" s="2" t="n"/>
-      <c r="C268" s="2" t="n"/>
+      <c r="B268" s="3" t="n"/>
+      <c r="C268" s="3" t="n"/>
     </row>
     <row r="269">
-      <c r="B269" s="2" t="n"/>
-      <c r="C269" s="2" t="n"/>
+      <c r="B269" s="3" t="n"/>
+      <c r="C269" s="3" t="n"/>
     </row>
     <row r="270">
-      <c r="B270" s="2" t="n"/>
-      <c r="C270" s="2" t="n"/>
+      <c r="B270" s="3" t="n"/>
+      <c r="C270" s="3" t="n"/>
     </row>
     <row r="271">
-      <c r="B271" s="2" t="n"/>
-      <c r="C271" s="2" t="n"/>
+      <c r="B271" s="3" t="n"/>
+      <c r="C271" s="3" t="n"/>
     </row>
     <row r="272">
-      <c r="B272" s="2" t="n"/>
-      <c r="C272" s="2" t="n"/>
+      <c r="B272" s="3" t="n"/>
+      <c r="C272" s="3" t="n"/>
     </row>
     <row r="273">
-      <c r="B273" s="2" t="n"/>
-      <c r="C273" s="2" t="n"/>
+      <c r="B273" s="3" t="n"/>
+      <c r="C273" s="3" t="n"/>
     </row>
     <row r="274">
-      <c r="B274" s="2" t="n"/>
-      <c r="C274" s="2" t="n"/>
+      <c r="B274" s="3" t="n"/>
+      <c r="C274" s="3" t="n"/>
     </row>
     <row r="275">
-      <c r="B275" s="2" t="n"/>
-      <c r="C275" s="2" t="n"/>
+      <c r="B275" s="3" t="n"/>
+      <c r="C275" s="3" t="n"/>
     </row>
     <row r="276">
-      <c r="B276" s="2" t="n"/>
-      <c r="C276" s="2" t="n"/>
+      <c r="B276" s="3" t="n"/>
+      <c r="C276" s="3" t="n"/>
     </row>
     <row r="277">
-      <c r="B277" s="2" t="n"/>
-      <c r="C277" s="2" t="n"/>
+      <c r="B277" s="3" t="n"/>
+      <c r="C277" s="3" t="n"/>
     </row>
     <row r="278">
-      <c r="B278" s="2" t="n"/>
-      <c r="C278" s="2" t="n"/>
+      <c r="B278" s="3" t="n"/>
+      <c r="C278" s="3" t="n"/>
     </row>
     <row r="279">
-      <c r="B279" s="2" t="n"/>
-      <c r="C279" s="2" t="n"/>
+      <c r="B279" s="3" t="n"/>
+      <c r="C279" s="3" t="n"/>
     </row>
     <row r="280">
-      <c r="B280" s="2" t="n"/>
-      <c r="C280" s="2" t="n"/>
+      <c r="B280" s="3" t="n"/>
+      <c r="C280" s="3" t="n"/>
     </row>
     <row r="281">
-      <c r="B281" s="2" t="n"/>
-      <c r="C281" s="2" t="n"/>
+      <c r="B281" s="3" t="n"/>
+      <c r="C281" s="3" t="n"/>
     </row>
     <row r="282">
-      <c r="B282" s="2" t="n"/>
-      <c r="C282" s="2" t="n"/>
+      <c r="B282" s="3" t="n"/>
+      <c r="C282" s="3" t="n"/>
     </row>
     <row r="283">
-      <c r="B283" s="2" t="n"/>
-      <c r="C283" s="2" t="n"/>
+      <c r="B283" s="3" t="n"/>
+      <c r="C283" s="3" t="n"/>
     </row>
     <row r="284">
-      <c r="B284" s="2" t="n"/>
-      <c r="C284" s="2" t="n"/>
+      <c r="B284" s="3" t="n"/>
+      <c r="C284" s="3" t="n"/>
     </row>
     <row r="285">
-      <c r="B285" s="2" t="n"/>
-      <c r="C285" s="2" t="n"/>
+      <c r="B285" s="3" t="n"/>
+      <c r="C285" s="3" t="n"/>
     </row>
     <row r="286">
-      <c r="B286" s="2" t="n"/>
-      <c r="C286" s="2" t="n"/>
+      <c r="B286" s="3" t="n"/>
+      <c r="C286" s="3" t="n"/>
     </row>
     <row r="287">
-      <c r="B287" s="2" t="n"/>
-      <c r="C287" s="2" t="n"/>
+      <c r="B287" s="3" t="n"/>
+      <c r="C287" s="3" t="n"/>
     </row>
     <row r="288">
-      <c r="B288" s="2" t="n"/>
-      <c r="C288" s="2" t="n"/>
+      <c r="B288" s="3" t="n"/>
+      <c r="C288" s="3" t="n"/>
     </row>
     <row r="289">
-      <c r="B289" s="2" t="n"/>
-      <c r="C289" s="2" t="n"/>
+      <c r="B289" s="3" t="n"/>
+      <c r="C289" s="3" t="n"/>
     </row>
     <row r="290">
-      <c r="B290" s="2" t="n"/>
-      <c r="C290" s="2" t="n"/>
+      <c r="B290" s="3" t="n"/>
+      <c r="C290" s="3" t="n"/>
     </row>
     <row r="291">
-      <c r="B291" s="2" t="n"/>
-      <c r="C291" s="2" t="n"/>
+      <c r="B291" s="3" t="n"/>
+      <c r="C291" s="3" t="n"/>
     </row>
     <row r="292">
-      <c r="B292" s="2" t="n"/>
-      <c r="C292" s="2" t="n"/>
+      <c r="B292" s="3" t="n"/>
+      <c r="C292" s="3" t="n"/>
     </row>
     <row r="293">
-      <c r="B293" s="2" t="n"/>
-      <c r="C293" s="2" t="n"/>
+      <c r="B293" s="3" t="n"/>
+      <c r="C293" s="3" t="n"/>
     </row>
     <row r="294">
-      <c r="B294" s="2" t="n"/>
-      <c r="C294" s="2" t="n"/>
+      <c r="B294" s="3" t="n"/>
+      <c r="C294" s="3" t="n"/>
     </row>
     <row r="295">
-      <c r="B295" s="2" t="n"/>
-      <c r="C295" s="2" t="n"/>
+      <c r="B295" s="3" t="n"/>
+      <c r="C295" s="3" t="n"/>
     </row>
     <row r="296">
-      <c r="B296" s="2" t="n"/>
-      <c r="C296" s="2" t="n"/>
+      <c r="B296" s="3" t="n"/>
+      <c r="C296" s="3" t="n"/>
     </row>
     <row r="297">
-      <c r="B297" s="2" t="n"/>
-      <c r="C297" s="2" t="n"/>
+      <c r="B297" s="3" t="n"/>
+      <c r="C297" s="3" t="n"/>
     </row>
     <row r="298">
-      <c r="B298" s="2" t="n"/>
-      <c r="C298" s="2" t="n"/>
+      <c r="B298" s="3" t="n"/>
+      <c r="C298" s="3" t="n"/>
     </row>
     <row r="299">
-      <c r="B299" s="2" t="n"/>
-      <c r="C299" s="2" t="n"/>
+      <c r="B299" s="3" t="n"/>
+      <c r="C299" s="3" t="n"/>
     </row>
     <row r="300">
-      <c r="B300" s="2" t="n"/>
-      <c r="C300" s="2" t="n"/>
+      <c r="B300" s="3" t="n"/>
+      <c r="C300" s="3" t="n"/>
     </row>
     <row r="301">
-      <c r="B301" s="2" t="n"/>
-      <c r="C301" s="2" t="n"/>
+      <c r="B301" s="3" t="n"/>
+      <c r="C301" s="3" t="n"/>
     </row>
     <row r="302">
-      <c r="B302" s="2" t="n"/>
-      <c r="C302" s="2" t="n"/>
+      <c r="B302" s="3" t="n"/>
+      <c r="C302" s="3" t="n"/>
     </row>
     <row r="303">
-      <c r="B303" s="2" t="n"/>
-      <c r="C303" s="2" t="n"/>
+      <c r="B303" s="3" t="n"/>
+      <c r="C303" s="3" t="n"/>
     </row>
     <row r="304">
-      <c r="B304" s="2" t="n"/>
-      <c r="C304" s="2" t="n"/>
+      <c r="B304" s="3" t="n"/>
+      <c r="C304" s="3" t="n"/>
     </row>
     <row r="305">
-      <c r="B305" s="2" t="n"/>
-      <c r="C305" s="2" t="n"/>
+      <c r="B305" s="3" t="n"/>
+      <c r="C305" s="3" t="n"/>
     </row>
     <row r="306">
-      <c r="B306" s="2" t="n"/>
-      <c r="C306" s="2" t="n"/>
+      <c r="B306" s="3" t="n"/>
+      <c r="C306" s="3" t="n"/>
     </row>
     <row r="307">
-      <c r="B307" s="2" t="n"/>
-      <c r="C307" s="2" t="n"/>
+      <c r="B307" s="3" t="n"/>
+      <c r="C307" s="3" t="n"/>
     </row>
     <row r="308">
-      <c r="B308" s="2" t="n"/>
-      <c r="C308" s="2" t="n"/>
+      <c r="B308" s="3" t="n"/>
+      <c r="C308" s="3" t="n"/>
     </row>
     <row r="309">
-      <c r="B309" s="2" t="n"/>
-      <c r="C309" s="2" t="n"/>
+      <c r="B309" s="3" t="n"/>
+      <c r="C309" s="3" t="n"/>
     </row>
     <row r="310">
-      <c r="B310" s="2" t="n"/>
-      <c r="C310" s="2" t="n"/>
+      <c r="B310" s="3" t="n"/>
+      <c r="C310" s="3" t="n"/>
     </row>
     <row r="311">
-      <c r="B311" s="2" t="n"/>
-      <c r="C311" s="2" t="n"/>
+      <c r="B311" s="3" t="n"/>
+      <c r="C311" s="3" t="n"/>
     </row>
     <row r="312">
-      <c r="B312" s="2" t="n"/>
-      <c r="C312" s="2" t="n"/>
+      <c r="B312" s="3" t="n"/>
+      <c r="C312" s="3" t="n"/>
     </row>
     <row r="313">
-      <c r="B313" s="2" t="n"/>
-      <c r="C313" s="2" t="n"/>
+      <c r="B313" s="3" t="n"/>
+      <c r="C313" s="3" t="n"/>
     </row>
     <row r="314">
-      <c r="B314" s="2" t="n"/>
-      <c r="C314" s="2" t="n"/>
+      <c r="B314" s="3" t="n"/>
+      <c r="C314" s="3" t="n"/>
     </row>
     <row r="315">
-      <c r="B315" s="2" t="n"/>
-      <c r="C315" s="2" t="n"/>
+      <c r="B315" s="3" t="n"/>
+      <c r="C315" s="3" t="n"/>
     </row>
     <row r="316">
-      <c r="B316" s="2" t="n"/>
-      <c r="C316" s="2" t="n"/>
+      <c r="B316" s="3" t="n"/>
+      <c r="C316" s="3" t="n"/>
     </row>
     <row r="317">
-      <c r="B317" s="2" t="n"/>
-      <c r="C317" s="2" t="n"/>
+      <c r="B317" s="3" t="n"/>
+      <c r="C317" s="3" t="n"/>
     </row>
     <row r="318">
-      <c r="B318" s="2" t="n"/>
-      <c r="C318" s="2" t="n"/>
+      <c r="B318" s="3" t="n"/>
+      <c r="C318" s="3" t="n"/>
     </row>
     <row r="319">
-      <c r="B319" s="2" t="n"/>
-      <c r="C319" s="2" t="n"/>
+      <c r="B319" s="3" t="n"/>
+      <c r="C319" s="3" t="n"/>
     </row>
     <row r="320">
-      <c r="B320" s="2" t="n"/>
-      <c r="C320" s="2" t="n"/>
+      <c r="B320" s="3" t="n"/>
+      <c r="C320" s="3" t="n"/>
     </row>
     <row r="321">
-      <c r="B321" s="2" t="n"/>
-      <c r="C321" s="2" t="n"/>
+      <c r="B321" s="3" t="n"/>
+      <c r="C321" s="3" t="n"/>
     </row>
     <row r="322">
-      <c r="B322" s="2" t="n"/>
-      <c r="C322" s="2" t="n"/>
+      <c r="B322" s="3" t="n"/>
+      <c r="C322" s="3" t="n"/>
     </row>
     <row r="323">
-      <c r="B323" s="2" t="n"/>
-      <c r="C323" s="2" t="n"/>
+      <c r="B323" s="3" t="n"/>
+      <c r="C323" s="3" t="n"/>
     </row>
     <row r="324">
-      <c r="B324" s="2" t="n"/>
-      <c r="C324" s="2" t="n"/>
+      <c r="B324" s="3" t="n"/>
+      <c r="C324" s="3" t="n"/>
     </row>
     <row r="325">
-      <c r="B325" s="2" t="n"/>
-      <c r="C325" s="2" t="n"/>
+      <c r="B325" s="3" t="n"/>
+      <c r="C325" s="3" t="n"/>
     </row>
     <row r="326">
-      <c r="B326" s="2" t="n"/>
-      <c r="C326" s="2" t="n"/>
+      <c r="B326" s="3" t="n"/>
+      <c r="C326" s="3" t="n"/>
     </row>
     <row r="327">
-      <c r="B327" s="2" t="n"/>
-      <c r="C327" s="2" t="n"/>
+      <c r="B327" s="3" t="n"/>
+      <c r="C327" s="3" t="n"/>
     </row>
     <row r="328">
-      <c r="B328" s="2" t="n"/>
-      <c r="C328" s="2" t="n"/>
+      <c r="B328" s="3" t="n"/>
+      <c r="C328" s="3" t="n"/>
     </row>
     <row r="329">
-      <c r="B329" s="2" t="n"/>
-      <c r="C329" s="2" t="n"/>
+      <c r="B329" s="3" t="n"/>
+      <c r="C329" s="3" t="n"/>
     </row>
     <row r="330">
-      <c r="B330" s="2" t="n"/>
-      <c r="C330" s="2" t="n"/>
+      <c r="B330" s="3" t="n"/>
+      <c r="C330" s="3" t="n"/>
     </row>
     <row r="331">
-      <c r="B331" s="2" t="n"/>
-      <c r="C331" s="2" t="n"/>
+      <c r="B331" s="3" t="n"/>
+      <c r="C331" s="3" t="n"/>
     </row>
     <row r="332">
-      <c r="B332" s="2" t="n"/>
-      <c r="C332" s="2" t="n"/>
+      <c r="B332" s="3" t="n"/>
+      <c r="C332" s="3" t="n"/>
     </row>
     <row r="333">
-      <c r="B333" s="2" t="n"/>
-      <c r="C333" s="2" t="n"/>
+      <c r="B333" s="3" t="n"/>
+      <c r="C333" s="3" t="n"/>
     </row>
     <row r="334">
-      <c r="B334" s="2" t="n"/>
-      <c r="C334" s="2" t="n"/>
+      <c r="B334" s="3" t="n"/>
+      <c r="C334" s="3" t="n"/>
     </row>
     <row r="335">
-      <c r="B335" s="2" t="n"/>
-      <c r="C335" s="2" t="n"/>
+      <c r="B335" s="3" t="n"/>
+      <c r="C335" s="3" t="n"/>
     </row>
     <row r="336">
-      <c r="B336" s="2" t="n"/>
-      <c r="C336" s="2" t="n"/>
+      <c r="B336" s="3" t="n"/>
+      <c r="C336" s="3" t="n"/>
     </row>
     <row r="337">
-      <c r="B337" s="2" t="n"/>
-      <c r="C337" s="2" t="n"/>
+      <c r="B337" s="3" t="n"/>
+      <c r="C337" s="3" t="n"/>
     </row>
     <row r="338">
-      <c r="B338" s="2" t="n"/>
-      <c r="C338" s="2" t="n"/>
+      <c r="B338" s="3" t="n"/>
+      <c r="C338" s="3" t="n"/>
     </row>
     <row r="339">
-      <c r="B339" s="2" t="n"/>
-      <c r="C339" s="2" t="n"/>
+      <c r="B339" s="3" t="n"/>
+      <c r="C339" s="3" t="n"/>
     </row>
     <row r="340">
-      <c r="B340" s="2" t="n"/>
-      <c r="C340" s="2" t="n"/>
+      <c r="B340" s="3" t="n"/>
+      <c r="C340" s="3" t="n"/>
     </row>
     <row r="341">
-      <c r="B341" s="2" t="n"/>
-      <c r="C341" s="2" t="n"/>
+      <c r="B341" s="3" t="n"/>
+      <c r="C341" s="3" t="n"/>
     </row>
     <row r="342">
-      <c r="B342" s="2" t="n"/>
-      <c r="C342" s="2" t="n"/>
+      <c r="B342" s="3" t="n"/>
+      <c r="C342" s="3" t="n"/>
     </row>
     <row r="343">
-      <c r="B343" s="2" t="n"/>
-      <c r="C343" s="2" t="n"/>
+      <c r="B343" s="3" t="n"/>
+      <c r="C343" s="3" t="n"/>
     </row>
     <row r="344">
-      <c r="B344" s="2" t="n"/>
-      <c r="C344" s="2" t="n"/>
+      <c r="B344" s="3" t="n"/>
+      <c r="C344" s="3" t="n"/>
     </row>
     <row r="345">
-      <c r="B345" s="2" t="n"/>
-      <c r="C345" s="2" t="n"/>
+      <c r="B345" s="3" t="n"/>
+      <c r="C345" s="3" t="n"/>
     </row>
     <row r="346">
-      <c r="B346" s="2" t="n"/>
-      <c r="C346" s="2" t="n"/>
+      <c r="B346" s="3" t="n"/>
+      <c r="C346" s="3" t="n"/>
     </row>
     <row r="347">
-      <c r="B347" s="2" t="n"/>
-      <c r="C347" s="2" t="n"/>
+      <c r="B347" s="3" t="n"/>
+      <c r="C347" s="3" t="n"/>
     </row>
     <row r="348">
-      <c r="B348" s="2" t="n"/>
-      <c r="C348" s="2" t="n"/>
+      <c r="B348" s="3" t="n"/>
+      <c r="C348" s="3" t="n"/>
     </row>
     <row r="349">
-      <c r="B349" s="2" t="n"/>
-      <c r="C349" s="2" t="n"/>
+      <c r="B349" s="3" t="n"/>
+      <c r="C349" s="3" t="n"/>
     </row>
     <row r="350">
-      <c r="B350" s="2" t="n"/>
-      <c r="C350" s="2" t="n"/>
+      <c r="B350" s="3" t="n"/>
+      <c r="C350" s="3" t="n"/>
     </row>
     <row r="351">
-      <c r="B351" s="2" t="n"/>
-      <c r="C351" s="2" t="n"/>
+      <c r="B351" s="3" t="n"/>
+      <c r="C351" s="3" t="n"/>
     </row>
     <row r="352">
-      <c r="B352" s="2" t="n"/>
-      <c r="C352" s="2" t="n"/>
+      <c r="B352" s="3" t="n"/>
+      <c r="C352" s="3" t="n"/>
     </row>
     <row r="353">
-      <c r="B353" s="2" t="n"/>
-      <c r="C353" s="2" t="n"/>
+      <c r="B353" s="3" t="n"/>
+      <c r="C353" s="3" t="n"/>
     </row>
     <row r="354">
-      <c r="B354" s="2" t="n"/>
-      <c r="C354" s="2" t="n"/>
+      <c r="B354" s="3" t="n"/>
+      <c r="C354" s="3" t="n"/>
     </row>
     <row r="355">
-      <c r="B355" s="2" t="n"/>
-      <c r="C355" s="2" t="n"/>
+      <c r="B355" s="3" t="n"/>
+      <c r="C355" s="3" t="n"/>
     </row>
     <row r="356">
-      <c r="B356" s="2" t="n"/>
-      <c r="C356" s="2" t="n"/>
+      <c r="B356" s="3" t="n"/>
+      <c r="C356" s="3" t="n"/>
     </row>
     <row r="357">
-      <c r="B357" s="2" t="n"/>
-      <c r="C357" s="2" t="n"/>
+      <c r="B357" s="3" t="n"/>
+      <c r="C357" s="3" t="n"/>
     </row>
     <row r="358">
-      <c r="B358" s="2" t="n"/>
-      <c r="C358" s="2" t="n"/>
+      <c r="B358" s="3" t="n"/>
+      <c r="C358" s="3" t="n"/>
     </row>
     <row r="359">
-      <c r="B359" s="2" t="n"/>
-      <c r="C359" s="2" t="n"/>
+      <c r="B359" s="3" t="n"/>
+      <c r="C359" s="3" t="n"/>
     </row>
     <row r="360">
-      <c r="B360" s="2" t="n"/>
-      <c r="C360" s="2" t="n"/>
+      <c r="B360" s="3" t="n"/>
+      <c r="C360" s="3" t="n"/>
     </row>
     <row r="361">
-      <c r="B361" s="2" t="n"/>
-      <c r="C361" s="2" t="n"/>
+      <c r="B361" s="3" t="n"/>
+      <c r="C361" s="3" t="n"/>
     </row>
     <row r="362">
-      <c r="B362" s="2" t="n"/>
-      <c r="C362" s="2" t="n"/>
+      <c r="B362" s="3" t="n"/>
+      <c r="C362" s="3" t="n"/>
     </row>
     <row r="363">
-      <c r="B363" s="2" t="n"/>
-      <c r="C363" s="2" t="n"/>
+      <c r="B363" s="3" t="n"/>
+      <c r="C363" s="3" t="n"/>
     </row>
     <row r="364">
-      <c r="B364" s="2" t="n"/>
-      <c r="C364" s="2" t="n"/>
+      <c r="B364" s="3" t="n"/>
+      <c r="C364" s="3" t="n"/>
     </row>
     <row r="365">
-      <c r="B365" s="2" t="n"/>
-      <c r="C365" s="2" t="n"/>
+      <c r="B365" s="3" t="n"/>
+      <c r="C365" s="3" t="n"/>
     </row>
     <row r="366">
-      <c r="B366" s="2" t="n"/>
-      <c r="C366" s="2" t="n"/>
+      <c r="B366" s="3" t="n"/>
+      <c r="C366" s="3" t="n"/>
     </row>
     <row r="367">
-      <c r="B367" s="2" t="n"/>
-      <c r="C367" s="2" t="n"/>
+      <c r="B367" s="3" t="n"/>
+      <c r="C367" s="3" t="n"/>
     </row>
     <row r="368">
-      <c r="B368" s="2" t="n"/>
-      <c r="C368" s="2" t="n"/>
+      <c r="B368" s="3" t="n"/>
+      <c r="C368" s="3" t="n"/>
     </row>
     <row r="369">
-      <c r="B369" s="2" t="n"/>
-      <c r="C369" s="2" t="n"/>
+      <c r="B369" s="3" t="n"/>
+      <c r="C369" s="3" t="n"/>
     </row>
     <row r="370">
-      <c r="B370" s="2" t="n"/>
-      <c r="C370" s="2" t="n"/>
+      <c r="B370" s="3" t="n"/>
+      <c r="C370" s="3" t="n"/>
     </row>
     <row r="371">
-      <c r="B371" s="2" t="n"/>
-      <c r="C371" s="2" t="n"/>
+      <c r="B371" s="3" t="n"/>
+      <c r="C371" s="3" t="n"/>
     </row>
     <row r="372">
-      <c r="B372" s="2" t="n"/>
-      <c r="C372" s="2" t="n"/>
+      <c r="B372" s="3" t="n"/>
+      <c r="C372" s="3" t="n"/>
     </row>
     <row r="373">
-      <c r="B373" s="2" t="n"/>
-      <c r="C373" s="2" t="n"/>
+      <c r="B373" s="3" t="n"/>
+      <c r="C373" s="3" t="n"/>
     </row>
     <row r="374">
-      <c r="B374" s="2" t="n"/>
-      <c r="C374" s="2" t="n"/>
+      <c r="B374" s="3" t="n"/>
+      <c r="C374" s="3" t="n"/>
     </row>
     <row r="375">
-      <c r="B375" s="2" t="n"/>
-      <c r="C375" s="2" t="n"/>
+      <c r="B375" s="3" t="n"/>
+      <c r="C375" s="3" t="n"/>
     </row>
     <row r="376">
-      <c r="B376" s="2" t="n"/>
-      <c r="C376" s="2" t="n"/>
+      <c r="B376" s="3" t="n"/>
+      <c r="C376" s="3" t="n"/>
     </row>
     <row r="377">
-      <c r="B377" s="2" t="n"/>
-      <c r="C377" s="2" t="n"/>
+      <c r="B377" s="3" t="n"/>
+      <c r="C377" s="3" t="n"/>
     </row>
     <row r="378">
-      <c r="B378" s="2" t="n"/>
-      <c r="C378" s="2" t="n"/>
+      <c r="B378" s="3" t="n"/>
+      <c r="C378" s="3" t="n"/>
     </row>
     <row r="379">
-      <c r="B379" s="2" t="n"/>
-      <c r="C379" s="2" t="n"/>
+      <c r="B379" s="3" t="n"/>
+      <c r="C379" s="3" t="n"/>
     </row>
     <row r="380">
-      <c r="B380" s="2" t="n"/>
-      <c r="C380" s="2" t="n"/>
+      <c r="B380" s="3" t="n"/>
+      <c r="C380" s="3" t="n"/>
     </row>
     <row r="381">
-      <c r="B381" s="2" t="n"/>
-      <c r="C381" s="2" t="n"/>
+      <c r="B381" s="3" t="n"/>
+      <c r="C381" s="3" t="n"/>
     </row>
     <row r="382">
-      <c r="B382" s="2" t="n"/>
-      <c r="C382" s="2" t="n"/>
+      <c r="B382" s="3" t="n"/>
+      <c r="C382" s="3" t="n"/>
     </row>
     <row r="383">
-      <c r="B383" s="2" t="n"/>
-      <c r="C383" s="2" t="n"/>
+      <c r="B383" s="3" t="n"/>
+      <c r="C383" s="3" t="n"/>
     </row>
     <row r="384">
-      <c r="B384" s="2" t="n"/>
-      <c r="C384" s="2" t="n"/>
+      <c r="B384" s="3" t="n"/>
+      <c r="C384" s="3" t="n"/>
     </row>
     <row r="385">
-      <c r="B385" s="2" t="n"/>
-      <c r="C385" s="2" t="n"/>
+      <c r="B385" s="3" t="n"/>
+      <c r="C385" s="3" t="n"/>
     </row>
     <row r="386">
-      <c r="B386" s="2" t="n"/>
-      <c r="C386" s="2" t="n"/>
+      <c r="B386" s="3" t="n"/>
+      <c r="C386" s="3" t="n"/>
     </row>
     <row r="387">
-      <c r="B387" s="2" t="n"/>
-      <c r="C387" s="2" t="n"/>
+      <c r="B387" s="3" t="n"/>
+      <c r="C387" s="3" t="n"/>
     </row>
     <row r="388">
-      <c r="B388" s="2" t="n"/>
-      <c r="C388" s="2" t="n"/>
+      <c r="B388" s="3" t="n"/>
+      <c r="C388" s="3" t="n"/>
     </row>
     <row r="389">
-      <c r="B389" s="2" t="n"/>
-      <c r="C389" s="2" t="n"/>
+      <c r="B389" s="3" t="n"/>
+      <c r="C389" s="3" t="n"/>
     </row>
     <row r="390">
-      <c r="B390" s="2" t="n"/>
-      <c r="C390" s="2" t="n"/>
+      <c r="B390" s="3" t="n"/>
+      <c r="C390" s="3" t="n"/>
     </row>
     <row r="391">
-      <c r="B391" s="2" t="n"/>
-      <c r="C391" s="2" t="n"/>
+      <c r="B391" s="3" t="n"/>
+      <c r="C391" s="3" t="n"/>
     </row>
     <row r="392">
-      <c r="B392" s="2" t="n"/>
-      <c r="C392" s="2" t="n"/>
+      <c r="B392" s="3" t="n"/>
+      <c r="C392" s="3" t="n"/>
     </row>
     <row r="393">
-      <c r="B393" s="2" t="n"/>
-      <c r="C393" s="2" t="n"/>
+      <c r="B393" s="3" t="n"/>
+      <c r="C393" s="3" t="n"/>
     </row>
     <row r="394">
-      <c r="B394" s="2" t="n"/>
-      <c r="C394" s="2" t="n"/>
+      <c r="B394" s="3" t="n"/>
+      <c r="C394" s="3" t="n"/>
     </row>
     <row r="395">
-      <c r="B395" s="2" t="n"/>
-      <c r="C395" s="2" t="n"/>
+      <c r="B395" s="3" t="n"/>
+      <c r="C395" s="3" t="n"/>
     </row>
     <row r="396">
-      <c r="B396" s="2" t="n"/>
-      <c r="C396" s="2" t="n"/>
+      <c r="B396" s="3" t="n"/>
+      <c r="C396" s="3" t="n"/>
     </row>
     <row r="397">
-      <c r="B397" s="2" t="n"/>
-      <c r="C397" s="2" t="n"/>
+      <c r="B397" s="3" t="n"/>
+      <c r="C397" s="3" t="n"/>
     </row>
     <row r="398">
-      <c r="B398" s="2" t="n"/>
-      <c r="C398" s="2" t="n"/>
+      <c r="B398" s="3" t="n"/>
+      <c r="C398" s="3" t="n"/>
     </row>
     <row r="399">
-      <c r="B399" s="2" t="n"/>
-      <c r="C399" s="2" t="n"/>
+      <c r="B399" s="3" t="n"/>
+      <c r="C399" s="3" t="n"/>
     </row>
     <row r="400">
-      <c r="B400" s="2" t="n"/>
-      <c r="C400" s="2" t="n"/>
+      <c r="B400" s="3" t="n"/>
+      <c r="C400" s="3" t="n"/>
     </row>
     <row r="401">
-      <c r="B401" s="2" t="n"/>
-      <c r="C401" s="2" t="n"/>
+      <c r="B401" s="3" t="n"/>
+      <c r="C401" s="3" t="n"/>
     </row>
     <row r="402">
-      <c r="B402" s="2" t="n"/>
-      <c r="C402" s="2" t="n"/>
+      <c r="B402" s="3" t="n"/>
+      <c r="C402" s="3" t="n"/>
     </row>
     <row r="403">
-      <c r="B403" s="2" t="n"/>
-      <c r="C403" s="2" t="n"/>
+      <c r="B403" s="3" t="n"/>
+      <c r="C403" s="3" t="n"/>
     </row>
     <row r="404">
-      <c r="B404" s="2" t="n"/>
-      <c r="C404" s="2" t="n"/>
+      <c r="B404" s="3" t="n"/>
+      <c r="C404" s="3" t="n"/>
     </row>
     <row r="405">
-      <c r="B405" s="2" t="n"/>
-      <c r="C405" s="2" t="n"/>
+      <c r="B405" s="3" t="n"/>
+      <c r="C405" s="3" t="n"/>
     </row>
     <row r="406">
-      <c r="B406" s="2" t="n"/>
-      <c r="C406" s="2" t="n"/>
+      <c r="B406" s="3" t="n"/>
+      <c r="C406" s="3" t="n"/>
     </row>
     <row r="407">
-      <c r="B407" s="2" t="n"/>
-      <c r="C407" s="2" t="n"/>
+      <c r="B407" s="3" t="n"/>
+      <c r="C407" s="3" t="n"/>
     </row>
     <row r="408">
-      <c r="B408" s="2" t="n"/>
-      <c r="C408" s="2" t="n"/>
+      <c r="B408" s="3" t="n"/>
+      <c r="C408" s="3" t="n"/>
     </row>
     <row r="409">
-      <c r="B409" s="2" t="n"/>
-      <c r="C409" s="2" t="n"/>
+      <c r="B409" s="3" t="n"/>
+      <c r="C409" s="3" t="n"/>
     </row>
     <row r="410">
-      <c r="B410" s="2" t="n"/>
-      <c r="C410" s="2" t="n"/>
+      <c r="B410" s="3" t="n"/>
+      <c r="C410" s="3" t="n"/>
     </row>
     <row r="411">
-      <c r="B411" s="2" t="n"/>
-      <c r="C411" s="2" t="n"/>
+      <c r="B411" s="3" t="n"/>
+      <c r="C411" s="3" t="n"/>
     </row>
     <row r="412">
-      <c r="B412" s="2" t="n"/>
-      <c r="C412" s="2" t="n"/>
+      <c r="B412" s="3" t="n"/>
+      <c r="C412" s="3" t="n"/>
     </row>
     <row r="413">
-      <c r="B413" s="2" t="n"/>
-      <c r="C413" s="2" t="n"/>
+      <c r="B413" s="3" t="n"/>
+      <c r="C413" s="3" t="n"/>
     </row>
     <row r="414">
-      <c r="B414" s="2" t="n"/>
-      <c r="C414" s="2" t="n"/>
+      <c r="B414" s="3" t="n"/>
+      <c r="C414" s="3" t="n"/>
     </row>
     <row r="415">
-      <c r="B415" s="2" t="n"/>
-      <c r="C415" s="2" t="n"/>
+      <c r="B415" s="3" t="n"/>
+      <c r="C415" s="3" t="n"/>
     </row>
     <row r="416">
-      <c r="B416" s="2" t="n"/>
-      <c r="C416" s="2" t="n"/>
+      <c r="B416" s="3" t="n"/>
+      <c r="C416" s="3" t="n"/>
     </row>
     <row r="417">
-      <c r="B417" s="2" t="n"/>
-      <c r="C417" s="2" t="n"/>
+      <c r="B417" s="3" t="n"/>
+      <c r="C417" s="3" t="n"/>
     </row>
     <row r="418">
-      <c r="B418" s="2" t="n"/>
-      <c r="C418" s="2" t="n"/>
+      <c r="B418" s="3" t="n"/>
+      <c r="C418" s="3" t="n"/>
     </row>
     <row r="419">
-      <c r="B419" s="2" t="n"/>
-      <c r="C419" s="2" t="n"/>
+      <c r="B419" s="3" t="n"/>
+      <c r="C419" s="3" t="n"/>
     </row>
     <row r="420">
-      <c r="B420" s="2" t="n"/>
-      <c r="C420" s="2" t="n"/>
+      <c r="B420" s="3" t="n"/>
+      <c r="C420" s="3" t="n"/>
     </row>
     <row r="421">
-      <c r="B421" s="2" t="n"/>
-      <c r="C421" s="2" t="n"/>
+      <c r="B421" s="3" t="n"/>
+      <c r="C421" s="3" t="n"/>
     </row>
     <row r="422">
-      <c r="B422" s="2" t="n"/>
-      <c r="C422" s="2" t="n"/>
+      <c r="B422" s="3" t="n"/>
+      <c r="C422" s="3" t="n"/>
     </row>
     <row r="423">
-      <c r="B423" s="2" t="n"/>
-      <c r="C423" s="2" t="n"/>
+      <c r="B423" s="3" t="n"/>
+      <c r="C423" s="3" t="n"/>
     </row>
     <row r="424">
-      <c r="B424" s="2" t="n"/>
-      <c r="C424" s="2" t="n"/>
+      <c r="B424" s="3" t="n"/>
+      <c r="C424" s="3" t="n"/>
     </row>
     <row r="425">
-      <c r="B425" s="2" t="n"/>
-      <c r="C425" s="2" t="n"/>
+      <c r="B425" s="3" t="n"/>
+      <c r="C425" s="3" t="n"/>
     </row>
     <row r="426">
-      <c r="B426" s="2" t="n"/>
-      <c r="C426" s="2" t="n"/>
+      <c r="B426" s="3" t="n"/>
+      <c r="C426" s="3" t="n"/>
     </row>
     <row r="427">
-      <c r="B427" s="2" t="n"/>
-      <c r="C427" s="2" t="n"/>
+      <c r="B427" s="3" t="n"/>
+      <c r="C427" s="3" t="n"/>
     </row>
     <row r="428">
-      <c r="B428" s="2" t="n"/>
-      <c r="C428" s="2" t="n"/>
+      <c r="B428" s="3" t="n"/>
+      <c r="C428" s="3" t="n"/>
     </row>
     <row r="429">
-      <c r="B429" s="2" t="n"/>
-      <c r="C429" s="2" t="n"/>
+      <c r="B429" s="3" t="n"/>
+      <c r="C429" s="3" t="n"/>
     </row>
     <row r="430">
-      <c r="B430" s="2" t="n"/>
-      <c r="C430" s="2" t="n"/>
+      <c r="B430" s="3" t="n"/>
+      <c r="C430" s="3" t="n"/>
     </row>
     <row r="431">
-      <c r="B431" s="2" t="n"/>
-      <c r="C431" s="2" t="n"/>
+      <c r="B431" s="3" t="n"/>
+      <c r="C431" s="3" t="n"/>
     </row>
     <row r="432">
-      <c r="B432" s="2" t="n"/>
-      <c r="C432" s="2" t="n"/>
+      <c r="B432" s="3" t="n"/>
+      <c r="C432" s="3" t="n"/>
     </row>
     <row r="433">
-      <c r="B433" s="2" t="n"/>
-      <c r="C433" s="2" t="n"/>
+      <c r="B433" s="3" t="n"/>
+      <c r="C433" s="3" t="n"/>
     </row>
     <row r="434">
-      <c r="B434" s="2" t="n"/>
-      <c r="C434" s="2" t="n"/>
+      <c r="B434" s="3" t="n"/>
+      <c r="C434" s="3" t="n"/>
     </row>
     <row r="435">
-      <c r="B435" s="2" t="n"/>
-      <c r="C435" s="2" t="n"/>
+      <c r="B435" s="3" t="n"/>
+      <c r="C435" s="3" t="n"/>
     </row>
     <row r="436">
-      <c r="B436" s="2" t="n"/>
-      <c r="C436" s="2" t="n"/>
+      <c r="B436" s="3" t="n"/>
+      <c r="C436" s="3" t="n"/>
     </row>
     <row r="437">
-      <c r="B437" s="2" t="n"/>
-      <c r="C437" s="2" t="n"/>
+      <c r="B437" s="3" t="n"/>
+      <c r="C437" s="3" t="n"/>
     </row>
     <row r="438">
-      <c r="B438" s="2" t="n"/>
-      <c r="C438" s="2" t="n"/>
+      <c r="B438" s="3" t="n"/>
+      <c r="C438" s="3" t="n"/>
     </row>
     <row r="439">
-      <c r="B439" s="2" t="n"/>
-      <c r="C439" s="2" t="n"/>
+      <c r="B439" s="3" t="n"/>
+      <c r="C439" s="3" t="n"/>
     </row>
     <row r="440">
-      <c r="B440" s="2" t="n"/>
-      <c r="C440" s="2" t="n"/>
+      <c r="B440" s="3" t="n"/>
+      <c r="C440" s="3" t="n"/>
     </row>
     <row r="441">
-      <c r="B441" s="2" t="n"/>
-      <c r="C441" s="2" t="n"/>
+      <c r="B441" s="3" t="n"/>
+      <c r="C441" s="3" t="n"/>
     </row>
     <row r="442">
-      <c r="B442" s="2" t="n"/>
-      <c r="C442" s="2" t="n"/>
+      <c r="B442" s="3" t="n"/>
+      <c r="C442" s="3" t="n"/>
     </row>
     <row r="443">
-      <c r="B443" s="2" t="n"/>
-      <c r="C443" s="2" t="n"/>
+      <c r="B443" s="3" t="n"/>
+      <c r="C443" s="3" t="n"/>
     </row>
     <row r="444">
-      <c r="B444" s="2" t="n"/>
-      <c r="C444" s="2" t="n"/>
+      <c r="B444" s="3" t="n"/>
+      <c r="C444" s="3" t="n"/>
     </row>
     <row r="445">
-      <c r="B445" s="2" t="n"/>
-      <c r="C445" s="2" t="n"/>
+      <c r="B445" s="3" t="n"/>
+      <c r="C445" s="3" t="n"/>
     </row>
     <row r="446">
-      <c r="B446" s="2" t="n"/>
-      <c r="C446" s="2" t="n"/>
+      <c r="B446" s="3" t="n"/>
+      <c r="C446" s="3" t="n"/>
     </row>
     <row r="447">
-      <c r="B447" s="2" t="n"/>
-      <c r="C447" s="2" t="n"/>
+      <c r="B447" s="3" t="n"/>
+      <c r="C447" s="3" t="n"/>
     </row>
     <row r="448">
-      <c r="B448" s="2" t="n"/>
-      <c r="C448" s="2" t="n"/>
+      <c r="B448" s="3" t="n"/>
+      <c r="C448" s="3" t="n"/>
     </row>
     <row r="449">
-      <c r="B449" s="2" t="n"/>
-      <c r="C449" s="2" t="n"/>
+      <c r="B449" s="3" t="n"/>
+      <c r="C449" s="3" t="n"/>
     </row>
     <row r="450">
-      <c r="B450" s="2" t="n"/>
-      <c r="C450" s="2" t="n"/>
+      <c r="B450" s="3" t="n"/>
+      <c r="C450" s="3" t="n"/>
     </row>
     <row r="451">
-      <c r="B451" s="2" t="n"/>
-      <c r="C451" s="2" t="n"/>
+      <c r="B451" s="3" t="n"/>
+      <c r="C451" s="3" t="n"/>
     </row>
     <row r="452">
-      <c r="B452" s="2" t="n"/>
-      <c r="C452" s="2" t="n"/>
+      <c r="B452" s="3" t="n"/>
+      <c r="C452" s="3" t="n"/>
     </row>
     <row r="453">
-      <c r="B453" s="2" t="n"/>
-      <c r="C453" s="2" t="n"/>
+      <c r="B453" s="3" t="n"/>
+      <c r="C453" s="3" t="n"/>
     </row>
     <row r="454">
-      <c r="B454" s="2" t="n"/>
-      <c r="C454" s="2" t="n"/>
+      <c r="B454" s="3" t="n"/>
+      <c r="C454" s="3" t="n"/>
     </row>
     <row r="455">
-      <c r="B455" s="2" t="n"/>
-      <c r="C455" s="2" t="n"/>
+      <c r="B455" s="3" t="n"/>
+      <c r="C455" s="3" t="n"/>
     </row>
     <row r="456">
-      <c r="B456" s="2" t="n"/>
-      <c r="C456" s="2" t="n"/>
+      <c r="B456" s="3" t="n"/>
+      <c r="C456" s="3" t="n"/>
     </row>
     <row r="457">
-      <c r="B457" s="2" t="n"/>
-      <c r="C457" s="2" t="n"/>
+      <c r="B457" s="3" t="n"/>
+      <c r="C457" s="3" t="n"/>
     </row>
     <row r="458">
-      <c r="B458" s="2" t="n"/>
-      <c r="C458" s="2" t="n"/>
+      <c r="B458" s="3" t="n"/>
+      <c r="C458" s="3" t="n"/>
     </row>
     <row r="459">
-      <c r="B459" s="2" t="n"/>
-      <c r="C459" s="2" t="n"/>
+      <c r="B459" s="3" t="n"/>
+      <c r="C459" s="3" t="n"/>
     </row>
     <row r="460">
-      <c r="B460" s="2" t="n"/>
-      <c r="C460" s="2" t="n"/>
+      <c r="B460" s="3" t="n"/>
+      <c r="C460" s="3" t="n"/>
     </row>
     <row r="461">
-      <c r="B461" s="2" t="n"/>
-      <c r="C461" s="2" t="n"/>
+      <c r="B461" s="3" t="n"/>
+      <c r="C461" s="3" t="n"/>
     </row>
     <row r="462">
-      <c r="B462" s="2" t="n"/>
-      <c r="C462" s="2" t="n"/>
+      <c r="B462" s="3" t="n"/>
+      <c r="C462" s="3" t="n"/>
     </row>
     <row r="463">
-      <c r="B463" s="2" t="n"/>
-      <c r="C463" s="2" t="n"/>
+      <c r="B463" s="3" t="n"/>
+      <c r="C463" s="3" t="n"/>
     </row>
     <row r="464">
-      <c r="B464" s="2" t="n"/>
-      <c r="C464" s="2" t="n"/>
+      <c r="B464" s="3" t="n"/>
+      <c r="C464" s="3" t="n"/>
     </row>
     <row r="465">
-      <c r="B465" s="2" t="n"/>
-      <c r="C465" s="2" t="n"/>
+      <c r="B465" s="3" t="n"/>
+      <c r="C465" s="3" t="n"/>
     </row>
     <row r="466">
-      <c r="B466" s="2" t="n"/>
-      <c r="C466" s="2" t="n"/>
+      <c r="B466" s="3" t="n"/>
+      <c r="C466" s="3" t="n"/>
     </row>
     <row r="467">
-      <c r="B467" s="2" t="n"/>
-      <c r="C467" s="2" t="n"/>
+      <c r="B467" s="3" t="n"/>
+      <c r="C467" s="3" t="n"/>
     </row>
     <row r="468">
-      <c r="B468" s="2" t="n"/>
-      <c r="C468" s="2" t="n"/>
+      <c r="B468" s="3" t="n"/>
+      <c r="C468" s="3" t="n"/>
     </row>
     <row r="469">
-      <c r="B469" s="2" t="n"/>
-      <c r="C469" s="2" t="n"/>
+      <c r="B469" s="3" t="n"/>
+      <c r="C469" s="3" t="n"/>
     </row>
     <row r="470">
-      <c r="B470" s="2" t="n"/>
-      <c r="C470" s="2" t="n"/>
+      <c r="B470" s="3" t="n"/>
+      <c r="C470" s="3" t="n"/>
     </row>
     <row r="471">
-      <c r="B471" s="2" t="n"/>
-      <c r="C471" s="2" t="n"/>
+      <c r="B471" s="3" t="n"/>
+      <c r="C471" s="3" t="n"/>
     </row>
     <row r="472">
-      <c r="B472" s="2" t="n"/>
-      <c r="C472" s="2" t="n"/>
+      <c r="B472" s="3" t="n"/>
+      <c r="C472" s="3" t="n"/>
     </row>
     <row r="473">
-      <c r="B473" s="2" t="n"/>
-      <c r="C473" s="2" t="n"/>
+      <c r="B473" s="3" t="n"/>
+      <c r="C473" s="3" t="n"/>
     </row>
     <row r="474">
-      <c r="B474" s="2" t="n"/>
-      <c r="C474" s="2" t="n"/>
+      <c r="B474" s="3" t="n"/>
+      <c r="C474" s="3" t="n"/>
     </row>
     <row r="475">
-      <c r="B475" s="2" t="n"/>
-      <c r="C475" s="2" t="n"/>
+      <c r="B475" s="3" t="n"/>
+      <c r="C475" s="3" t="n"/>
     </row>
     <row r="476">
-      <c r="B476" s="2" t="n"/>
-      <c r="C476" s="2" t="n"/>
+      <c r="B476" s="3" t="n"/>
+      <c r="C476" s="3" t="n"/>
     </row>
     <row r="477">
-      <c r="B477" s="2" t="n"/>
-      <c r="C477" s="2" t="n"/>
+      <c r="B477" s="3" t="n"/>
+      <c r="C477" s="3" t="n"/>
     </row>
     <row r="478">
-      <c r="B478" s="2" t="n"/>
-      <c r="C478" s="2" t="n"/>
+      <c r="B478" s="3" t="n"/>
+      <c r="C478" s="3" t="n"/>
     </row>
     <row r="479">
-      <c r="B479" s="2" t="n"/>
-      <c r="C479" s="2" t="n"/>
+      <c r="B479" s="3" t="n"/>
+      <c r="C479" s="3" t="n"/>
     </row>
     <row r="480">
-      <c r="B480" s="2" t="n"/>
-      <c r="C480" s="2" t="n"/>
+      <c r="B480" s="3" t="n"/>
+      <c r="C480" s="3" t="n"/>
     </row>
     <row r="481">
-      <c r="B481" s="2" t="n"/>
-      <c r="C481" s="2" t="n"/>
+      <c r="B481" s="3" t="n"/>
+      <c r="C481" s="3" t="n"/>
     </row>
     <row r="482">
-      <c r="B482" s="2" t="n"/>
-      <c r="C482" s="2" t="n"/>
+      <c r="B482" s="3" t="n"/>
+      <c r="C482" s="3" t="n"/>
     </row>
     <row r="483">
-      <c r="B483" s="2" t="n"/>
-      <c r="C483" s="2" t="n"/>
+      <c r="B483" s="3" t="n"/>
+      <c r="C483" s="3" t="n"/>
     </row>
     <row r="484">
-      <c r="B484" s="2" t="n"/>
-      <c r="C484" s="2" t="n"/>
+      <c r="B484" s="3" t="n"/>
+      <c r="C484" s="3" t="n"/>
     </row>
     <row r="485">
-      <c r="B485" s="2" t="n"/>
-      <c r="C485" s="2" t="n"/>
+      <c r="B485" s="3" t="n"/>
+      <c r="C485" s="3" t="n"/>
     </row>
     <row r="486">
-      <c r="B486" s="2" t="n"/>
-      <c r="C486" s="2" t="n"/>
+      <c r="B486" s="3" t="n"/>
+      <c r="C486" s="3" t="n"/>
     </row>
     <row r="487">
-      <c r="B487" s="2" t="n"/>
-      <c r="C487" s="2" t="n"/>
+      <c r="B487" s="3" t="n"/>
+      <c r="C487" s="3" t="n"/>
     </row>
     <row r="488">
-      <c r="B488" s="2" t="n"/>
-      <c r="C488" s="2" t="n"/>
+      <c r="B488" s="3" t="n"/>
+      <c r="C488" s="3" t="n"/>
     </row>
     <row r="489">
-      <c r="B489" s="2" t="n"/>
-      <c r="C489" s="2" t="n"/>
+      <c r="B489" s="3" t="n"/>
+      <c r="C489" s="3" t="n"/>
     </row>
     <row r="490">
-      <c r="B490" s="2" t="n"/>
-      <c r="C490" s="2" t="n"/>
+      <c r="B490" s="3" t="n"/>
+      <c r="C490" s="3" t="n"/>
     </row>
     <row r="491">
-      <c r="B491" s="2" t="n"/>
-      <c r="C491" s="2" t="n"/>
+      <c r="B491" s="3" t="n"/>
+      <c r="C491" s="3" t="n"/>
     </row>
     <row r="492">
-      <c r="B492" s="2" t="n"/>
-      <c r="C492" s="2" t="n"/>
+      <c r="B492" s="3" t="n"/>
+      <c r="C492" s="3" t="n"/>
     </row>
     <row r="493">
-      <c r="B493" s="2" t="n"/>
-      <c r="C493" s="2" t="n"/>
+      <c r="B493" s="3" t="n"/>
+      <c r="C493" s="3" t="n"/>
     </row>
     <row r="494">
-      <c r="B494" s="2" t="n"/>
-      <c r="C494" s="2" t="n"/>
+      <c r="B494" s="3" t="n"/>
+      <c r="C494" s="3" t="n"/>
     </row>
     <row r="495">
-      <c r="B495" s="2" t="n"/>
-      <c r="C495" s="2" t="n"/>
+      <c r="B495" s="3" t="n"/>
+      <c r="C495" s="3" t="n"/>
     </row>
     <row r="496">
-      <c r="B496" s="2" t="n"/>
-      <c r="C496" s="2" t="n"/>
+      <c r="B496" s="3" t="n"/>
+      <c r="C496" s="3" t="n"/>
     </row>
     <row r="497">
-      <c r="B497" s="2" t="n"/>
-      <c r="C497" s="2" t="n"/>
+      <c r="B497" s="3" t="n"/>
+      <c r="C497" s="3" t="n"/>
     </row>
     <row r="498">
-      <c r="B498" s="2" t="n"/>
-      <c r="C498" s="2" t="n"/>
+      <c r="B498" s="3" t="n"/>
+      <c r="C498" s="3" t="n"/>
     </row>
     <row r="499">
-      <c r="B499" s="2" t="n"/>
-      <c r="C499" s="2" t="n"/>
+      <c r="B499" s="3" t="n"/>
+      <c r="C499" s="3" t="n"/>
     </row>
     <row r="500">
-      <c r="B500" s="2" t="n"/>
-      <c r="C500" s="2" t="n"/>
+      <c r="B500" s="3" t="n"/>
+      <c r="C500" s="3" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -5116,10 +5131,10 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>46300.25</v>
+        <v>46300</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>46302.91666666666</v>
+        <v>46302</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5147,10 +5162,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>46307.29166666666</v>
+        <v>46307</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46307.66666666666</v>
+        <v>46307</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -7173,14 +7188,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Terminübersicht – so wird sie ausgefüllt</t>
         </is>
@@ -7188,7 +7203,7 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Blatt „Termine“ – hier wird alles eingetragen</t>
         </is>
@@ -7218,202 +7233,245 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>D  Von       – Datum und Uhrzeit, z. B. 16.11.2026 08:00</t>
+          <t>D  Von       – nur Datum, z. B. 16.11.2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>E  Bis       – Datum und Uhrzeit, bei „Info“ darf das Feld leer bleiben</t>
+          <t>E  Bis       – nur Datum, bei „Info“ darf das Feld leer bleiben</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>F  Info      – kurze Beschreibung</t>
+          <t xml:space="preserve">              Uhrzeiten gehören NICHT hierher, sondern ins Blatt „Zeiten“.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
+          <t>F  Info      – kurze Beschreibung</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
           <t>G  Status    – offen / abgeschlossen / storniert</t>
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="B12" s="5" t="inlineStr">
+    <row r="12"/>
+    <row r="13">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Die Spalten Art, Prüfstand, Status und Termin-Nr haben ein Drop-Down:</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="5" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>in die Zelle klicken, dann rechts am Zellrand auf den Pfeil klicken.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="5" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>So kann kein Tippfehler und kein unbekannter Prüfstand entstehen.</t>
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Wann ist das Blatt „Zeiten“ nötig?</t>
-        </is>
-      </c>
-    </row>
+    <row r="16"/>
     <row r="17">
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Nur wenn der Prüfstand NICHT durchgehend außer Betrieb ist.</t>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Blatt „Zeiten“ – hier stehen die Uhrzeiten</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
-          <t>Beispiel: Kalibrierung von Montag bis Samstag, aber täglich nur 4–8 Stunden,</t>
+          <t>Das Blatt „Termine“ kennt nur ganze Tage. Sobald eine Uhrzeit eine Rolle</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>und zwischendurch zwei Tage gar nicht.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20"/>
+          <t>spielt, wird sie hier eingetragen – als Zeitraum mit Von und Bis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Ein Termin kann mehrere Zeilen haben (z. B. eine Kalibrierung, die über</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>Dann für jeden Zeitraum, in dem wirklich gearbeitet wurde, eine Zeile:</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Termin-Nr | Von | Bis | Notiz</t>
-        </is>
-      </c>
-    </row>
-    <row r="23"/>
+          <t>mehrere Tage läuft, aber täglich nur vormittags).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Wann ist das Blatt „Zeiten“ nötig?</t>
+        </is>
+      </c>
+    </row>
     <row r="24">
       <c r="B24" t="inlineStr">
         <is>
-          <t>Kein Eintrag im Blatt „Zeiten“ = Prüfstand war durchgehend außer Betrieb.</t>
+          <t>Nur wenn der Prüfstand NICHT durchgehend außer Betrieb ist.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>Bei Wartung und Ausfall ist das der Normalfall – das Blatt bleibt dann leer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
+          <t>Beispiel: Kalibrierung von Montag bis Samstag, aber täglich nur 4–8 Stunden,</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>und zwischendurch zwei Tage gar nicht.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>offen         – Termin läuft bzw. steht noch aus, wird am Kiosk angezeigt</t>
+          <t>Dann für jeden Zeitraum, in dem wirklich gearbeitet wurde, eine Zeile:</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Termin-Nr | Von | Bis | Notiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Kein Eintrag im Blatt „Zeiten“ = Prüfstand war durchgehend außer Betrieb.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Bei Wartung und Ausfall ist das der Normalfall – das Blatt bleibt dann leer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34">
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>offen         – Termin läuft bzw. steht noch aus, wird am Kiosk angezeigt</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
           <t>abgeschlossen – erledigt, geht in die Historie und in die Ausfallstatistik</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>storniert     – versehentlich eingetragen, zählt NICHT als Ausfall</t>
-        </is>
-      </c>
-    </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Nach dem Abschluss</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Abgeschlossene Zeilen aus „Termine“ in das Blatt „Archiv“ verschieben.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Die Historie bleibt im Gerät erhalten, auch wenn die Zeile hier verschwindet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35"/>
-    <row r="36">
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>Neue Prüfstände</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" t="inlineStr">
         <is>
-          <t>Im Blatt „Prüfstände“ unten eine Zeile ergänzen (Kennung, Bezeichnung, Auswahl).</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Das Dropdown im Blatt „Termine“ zieht automatisch nach.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39"/>
+          <t>storniert     – versehentlich eingetragen, zählt NICHT als Ausfall</t>
+        </is>
+      </c>
+    </row>
+    <row r="38"/>
+    <row r="39">
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Nach dem Abschluss</t>
+        </is>
+      </c>
+    </row>
     <row r="40">
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>Beispiele</t>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Abgeschlossene Zeilen aus „Termine“ in das Blatt „Archiv“ verschieben.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
+          <t>Die Historie bleibt im Gerät erhalten, auch wenn die Zeile hier verschwindet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42"/>
+    <row r="43">
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Neue Prüfstände</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Im Blatt „Prüfstände“ unten eine Zeile ergänzen (Kennung, Bezeichnung, Auswahl).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Das Dropdown im Blatt „Termine“ zieht automatisch nach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46"/>
+    <row r="47">
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Beispiele</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="inlineStr">
+        <is>
           <t>Die Zeilen in dieser Vorlage sind Muster zum Ansehen. Vor dem ersten</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="B42" t="inlineStr">
+    <row r="49">
+      <c r="B49" t="inlineStr">
         <is>
           <t>echten Eintrag löschen – sonst werden sie als echte Termine importiert.</t>
         </is>

</xml_diff>

<commit_message>
fix(excel): Zeiten-Blatt bleibt leer
Beispielbloecke im Blatt 'Zeiten' waeren als echte Ausfallzeiten importiert
worden - 22 statt 4 Stunden, je nachdem was in der Vorlage stand. Das Blatt
hat jetzt nur die Kopfzeile und das Dropdown.

Die Blocklogik pruefen eigene Testdateien statt der Vorlage: Kalibrierung ueber
sechs Kalendertage sind fuenf Werktage (83,75 h), ein Halbtag entsteht nur
durch einen Block (9:00-13:00 = 4 h).
</commit_message>
<xml_diff>
--- a/terminboard/vorlagen/termine_modell2.xlsx
+++ b/terminboard/vorlagen/termine_modell2.xlsx
@@ -22,11 +22,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="167" formatCode="DD.MM.YYYY HH:MM"/>
+    <numFmt numFmtId="166" formatCode="DD.MM.YYYY HH:MM"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -94,7 +93,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2785,16 +2784,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I500"/>
+  <dimension ref="A1:D500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="3" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2818,169 +2814,42 @@
           <t>Notiz</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Beispiel</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B2" s="6" t="n">
-        <v>46350.375</v>
-      </c>
-      <c r="C2" s="6" t="n">
-        <v>46350.54166666666</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Halbtag, Rest des Tages freigegeben</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>Halbtag: 09:00–13:00</t>
-        </is>
-      </c>
+      <c r="B2" s="6" t="n"/>
+      <c r="C2" s="6" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="6" t="n">
-        <v>46342.33333333334</v>
-      </c>
-      <c r="C3" s="6" t="n">
-        <v>46342.5</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Tag 1, vormittags</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>erster Block einer mehrtägigen</t>
-        </is>
-      </c>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="6" t="n">
-        <v>46343.33333333334</v>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>46343.66666666666</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Tag 2, ganztags</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr"/>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>Kalibrierung</t>
-        </is>
-      </c>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="6" t="n">
-        <v>46345.29166666666</v>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>46345.45833333334</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Tag 4, vormittags</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr"/>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>46346.33333333334</v>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>46346.58333333334</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Tag 5, 6 Stunden</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>Uhrzeiten</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>gehören ausschließlich</t>
-        </is>
-      </c>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="6" t="n"/>
-      <c r="H7" s="4" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>in dieses Blatt</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
-      <c r="H8" s="4" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>Kein Eintrag</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>Prüfstand war durchgehend</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="B10" s="6" t="n"/>
       <c r="C10" s="6" t="n"/>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>außer Betrieb</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="B11" s="6" t="n"/>

</xml_diff>

<commit_message>
feat(excel): Status farbig, echte Termine, Archiv leer
- Status offen rot, abgeschlossen gruen, storniert grau (bedingte
  Formatierung, gilt weiter wenn jemand den Wert aendert)
- Die vier laufenden Kalibrierungen stehen in der Vorlage
- Belastungsbank AHH in die Stammliste: ohne P-Nummer und anders herum
  geschrieben als die uebrigen, deshalb mit eigener Auswahl-Spalte
- Archiv bleibt leer, das fuellt das Geraet
- Tests haengen nicht mehr an festen Zahlen der Vorlage: die gehoert dem
  Betrieb und aendert sich
</commit_message>
<xml_diff>
--- a/terminboard/vorlagen/termine_modell2.xlsx
+++ b/terminboard/vorlagen/termine_modell2.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Anleitung" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="Pruefstaende">'Prüfstände'!$C$2:$C$16</definedName>
+    <definedName name="Pruefstaende">'Prüfstände'!$C$2:$C$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -101,6 +101,42 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+          <bgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00595959"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E7E6E6"/>
+          <bgColor rgb="00E7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -514,7 +550,7 @@
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>Beispiel</t>
+          <t>Legende</t>
         </is>
       </c>
     </row>
@@ -524,38 +560,38 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Wartung</t>
+          <t>Kalibrierung</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>P03 NRA</t>
+          <t>P11 PUMO HYCOM</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46328</v>
+        <v>46314</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>46328</v>
+        <v>46321</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Jahreswartung Hydraulik</t>
+          <t>Kalibrierung Hycom (Kristin + Glen) 07:00 - 14:00</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>abgeschlossen</t>
+          <t>offen</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>offen</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Wartung, erledigt</t>
+          <t>Prüfstand steht still (rot)</t>
         </is>
       </c>
     </row>
@@ -570,33 +606,33 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>P10 PTU TESTFUCHS</t>
+          <t>Belastungsbank AHH</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46342</v>
+        <v>46321</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>46347</v>
+        <v>46322</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Kalibrierung Druckmessung, unterbrochen</t>
+          <t>Kalibrierung (Sven + Glen) 15:00 - 22:00</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
           <t>abgeschlossen</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Kalibrierung über mehrere Tage –</t>
+          <t>erledigt (grün)</t>
         </is>
       </c>
     </row>
@@ -606,23 +642,21 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ausfall</t>
+          <t>Kalibrierung</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>P21 NRC HYCOM</t>
+          <t>P43 LOW-PRESSURE</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46344</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>46345</v>
-      </c>
+        <v>46331</v>
+      </c>
+      <c r="E4" s="3" t="n"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Steuerung ausgefallen, Ersatzteil</t>
+          <t>Kalibrierung (Kristin) 07:00 - 13:00</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -630,10 +664,14 @@
           <t>offen</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>storniert</t>
+        </is>
+      </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Zeitblöcke im Blatt „Zeiten“</t>
+          <t>zählt nicht (grau)</t>
         </is>
       </c>
     </row>
@@ -652,14 +690,14 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46350</v>
+        <v>46335</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>46350</v>
+        <v>46346</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Halbtag, Rest des Tages freigegeben</t>
+          <t>Kalibrierung (Bernd + Tommy) 08:00 - 15:00</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -667,152 +705,80 @@
           <t>offen</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>Info – „Bis“ darf leer bleiben</t>
-        </is>
-      </c>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Audit</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>P40 AKKU/HOCHDRUCK-RAUM</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>46353</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>46353</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>interner Audit</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr"/>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="3" t="n"/>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Von / Bis</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>nur Datum, keine Uhrzeit</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Info</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>P07 EHSV NRA</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>46357</v>
-      </c>
+      <c r="D7" s="3" t="n"/>
       <c r="E7" s="3" t="n"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Hinweis Software-Update</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>Von / Bis</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>nur Datum, keine Uhrzeit</t>
-        </is>
-      </c>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="D8" s="3" t="n"/>
       <c r="E8" s="3" t="n"/>
-      <c r="H8" s="4" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Uhrzeiten</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>gehören ins Blatt „Zeiten“</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="D9" s="3" t="n"/>
       <c r="E9" s="3" t="n"/>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>Art</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>Kalibrierung / Wartung /</t>
-        </is>
-      </c>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="D10" s="3" t="n"/>
       <c r="E10" s="3" t="n"/>
-      <c r="H10" s="4" t="inlineStr"/>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>Ausfall / Audit / Info</t>
+          <t>Kalibrierung / Wartung /</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="D11" s="3" t="n"/>
       <c r="E11" s="3" t="n"/>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>Prüfstand</t>
-        </is>
-      </c>
+      <c r="H11" s="4" t="inlineStr"/>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Reihenfolge: erst mit</t>
+          <t>Ausfall / Audit / Info</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="D12" s="3" t="n"/>
       <c r="E12" s="3" t="n"/>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>Dropdown wählen – falsche</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="D13" s="3" t="n"/>
       <c r="E13" s="3" t="n"/>
-      <c r="H13" s="4" t="inlineStr"/>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>Namen zählen nicht</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="D14" s="3" t="n"/>
@@ -2763,6 +2729,17 @@
       <c r="E500" s="3" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="G2:G500">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"offen"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"abgeschlossen"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"storniert"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiger Wert" error="Bitte einen Wert aus der Liste wählen." promptTitle="Art" prompt="Art des Termins wählen." type="list">
       <formula1>"Kalibrierung,Wartung,Ausfall,Audit,Info"</formula1>
@@ -4827,7 +4804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5104,6 +5081,23 @@
       <c r="C16" t="inlineStr">
         <is>
           <t>P43 LOW-PRESSURE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>AHH</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Belastungsbank</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Belastungsbank AHH</t>
         </is>
       </c>
     </row>
@@ -5168,66 +5162,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Ausfall</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>P02 NRA</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>46300</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>46302</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Kühlmittelverlust, Reparatur</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>abgeschlossen</t>
-        </is>
-      </c>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>8</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Wartung</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>P41 MIL</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>46307</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>46307</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Dichtungen getauscht</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>abgeschlossen</t>
-        </is>
-      </c>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="D4" s="3" t="n"/>
@@ -7218,6 +7158,17 @@
       <c r="E500" s="3" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="G2:G500">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"offen"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"abgeschlossen"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"storniert"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiger Wert" error="Bitte einen Wert aus der Liste wählen." promptTitle="Art" prompt="Art des Termins wählen." type="list">
       <formula1>"Kalibrierung,Wartung,Ausfall,Audit,Info"</formula1>

</xml_diff>

<commit_message>
feat(archiv): abgeschlossene Termine wandern von selbst ins Archiv
Nach dem Import verschiebt das Geraet Zeilen mit Status 'abgeschlossen' ins
Blatt 'Archiv' und loescht sie aus 'Termine'. Nummern bleiben, keine
Leerzeilen, Sicherung als .bak vor dem Schreiben; bei Fehler wird
zurueckgerollt. Das braucht Schreibrecht auf dem Stick - ist er nur lesend,
bleibt der Import gueltig und der Bericht sagt es.

Ausserdem: Die Zeitbloecke der vier laufenden Kalibrierungen stehen jetzt im
Blatt 'Zeiten'. Damit rechnet die Statistik 132 h statt 318 h.
</commit_message>
<xml_diff>
--- a/terminboard/vorlagen/termine_modell2.xlsx
+++ b/terminboard/vorlagen/termine_modell2.xlsx
@@ -22,10 +22,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
-    <numFmt numFmtId="166" formatCode="DD.MM.YYYY HH:MM"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="DD.MM.YYYY HH:MM"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -76,7 +77,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -552,7 +553,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Kalibrierung Hycom (Kristin + Glen) 07:00 - 14:00</t>
+          <t>Hycom, Kristin + Glen</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -583,7 +584,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Kalibrierung (Sven + Glen) 15:00 - 22:00</t>
+          <t>Belastungsbank, Sven + Glen</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -612,7 +613,7 @@
       <c r="E4" s="2" t="n"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Kalibrierung (Kristin) 07:00 - 13:00</t>
+          <t>Low-Pressure, Kristin</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -643,7 +644,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Kalibrierung (Bernd + Tommy) 08:00 - 15:00</t>
+          <t>THSA, Bernd + Tommy</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -4182,80 +4183,232 @@
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>46314.29166666666</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>46314.58333333334</v>
+      </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>46315.29166666666</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>46315.58333333334</v>
+      </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>46316.29166666666</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>46316.58333333334</v>
+      </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>46317.29166666666</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>46317.58333333334</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>46318.29166666666</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>46318.58333333334</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>46321.29166666666</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>46321.58333333334</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
+      <c r="A8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>46321.625</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>46321.91666666666</v>
+      </c>
+      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
+      <c r="A9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>46322.625</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>46322.91666666666</v>
+      </c>
+      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
+      <c r="A10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>46331.29166666666</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>46331.54166666666</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
+      <c r="A11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>46335.33333333334</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>46335.625</v>
+      </c>
+      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
+      <c r="A12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>46336.33333333334</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>46336.625</v>
+      </c>
+      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
+      <c r="A13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>46337.33333333334</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>46337.625</v>
+      </c>
+      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
+      <c r="A14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>46338.33333333334</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>46338.625</v>
+      </c>
+      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
+      <c r="A15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>46339.33333333334</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>46339.625</v>
+      </c>
+      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
+      <c r="A16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>46342.33333333334</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>46342.625</v>
+      </c>
+      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
+      <c r="A17" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>46343.33333333334</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>46343.625</v>
+      </c>
+      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="B18" s="3" t="n"/>
-      <c r="C18" s="3" t="n"/>
+      <c r="A18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>46344.33333333334</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>46344.625</v>
+      </c>
+      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
+      <c r="A19" t="n">
+        <v>4</v>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>46345.33333333334</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>46345.625</v>
+      </c>
+      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="n"/>
+      <c r="A20" t="n">
+        <v>4</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>46346.33333333334</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>46346.625</v>
+      </c>
+      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="B21" s="3" t="n"/>

</xml_diff>